<commit_message>
Actualizo discos 15 2 26
</commit_message>
<xml_diff>
--- a/public/discos.xlsx
+++ b/public/discos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="131">
   <si>
     <t>Artista</t>
   </si>
@@ -310,6 +310,483 @@
         <rFont val="Helvetica Neue"/>
       </rPr>
       <t>https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b</t>
+    </r>
+  </si>
+  <si>
+    <t>Green day</t>
+  </si>
+  <si>
+    <t>American Idiot</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279</t>
+    </r>
+  </si>
+  <si>
+    <t>David Guetta</t>
+  </si>
+  <si>
+    <t>Nothing but the beat</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7</t>
+    </r>
+  </si>
+  <si>
+    <t>Harrison George</t>
+  </si>
+  <si>
+    <t>Lo mejor de George Harrison</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg</t>
+    </r>
+  </si>
+  <si>
+    <t>Kool &amp; the Gang</t>
+  </si>
+  <si>
+    <t>Celebrate!</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473</t>
+    </r>
+  </si>
+  <si>
+    <t>Lali</t>
+  </si>
+  <si>
+    <t>No vayas a atender cuando el demonio llama</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4</t>
+    </r>
+  </si>
+  <si>
+    <t>Led Zeppelin</t>
+  </si>
+  <si>
+    <t>Led Zeppelin I</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f</t>
+    </r>
+  </si>
+  <si>
+    <t>Miguel Luis</t>
+  </si>
+  <si>
+    <t>Aries</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff</t>
+    </r>
+  </si>
+  <si>
+    <t>Busca una mujer</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca</t>
+    </r>
+  </si>
+  <si>
+    <t>Miranda!</t>
+  </si>
+  <si>
+    <t>Nuevo Hotel Miranda!</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e</t>
+    </r>
+  </si>
+  <si>
+    <t>Muse</t>
+  </si>
+  <si>
+    <t>Black Holes and Revelation</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400</t>
+    </r>
+  </si>
+  <si>
+    <t>No te Va Gustar</t>
+  </si>
+  <si>
+    <t>El calor del pleno invierno</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08</t>
+    </r>
+  </si>
+  <si>
+    <t>Por lo menos hoy</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3</t>
+    </r>
+  </si>
+  <si>
+    <t>Palito Ortega</t>
+  </si>
+  <si>
+    <t>Palito Ortega Nº 21</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135</t>
+    </r>
+  </si>
+  <si>
+    <t>Queen</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87</t>
+    </r>
+  </si>
+  <si>
+    <t>A Kind of Magic</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419</t>
+    </r>
+  </si>
+  <si>
+    <t>A Night at the Opera</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537</t>
+    </r>
+  </si>
+  <si>
+    <t>Flashgordon</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02</t>
+    </r>
+  </si>
+  <si>
+    <t>Ramones</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2733935c39bea149ac15c83c41a</t>
+    </r>
+  </si>
+  <si>
+    <t>Rodriguez Los</t>
+  </si>
+  <si>
+    <t>Hasta Luego</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2730320739a960dd4821b2aeaf1</t>
+    </r>
+  </si>
+  <si>
+    <t>Sin Documentos</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273139d10e0ae979a7b4a811140</t>
+    </r>
+  </si>
+  <si>
+    <t>Sanz Alejandro</t>
+  </si>
+  <si>
+    <t>Más</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2733443d9c76e9713a5986c983c</t>
+    </r>
+  </si>
+  <si>
+    <t>Silvestre y la Naranja</t>
+  </si>
+  <si>
+    <t>Alter Ego</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273dfc72dec3da479c81c575551</t>
+    </r>
+  </si>
+  <si>
+    <t>Soda Stereo</t>
+  </si>
+  <si>
+    <t>Canción Animal</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273c3780b28120b1bc2869a2ca7</t>
+    </r>
+  </si>
+  <si>
+    <t>Doble Vida</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2737e553e1367924fa3429a692c</t>
+    </r>
+  </si>
+  <si>
+    <t>Nada Personal</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e28947f6ad2f100af9c1965a</t>
+    </r>
+  </si>
+  <si>
+    <t>Signos</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273d8abc667a17dab2e1a6bd44e</t>
+    </r>
+  </si>
+  <si>
+    <t>Sosa Julio</t>
+  </si>
+  <si>
+    <t>Asi cantaba Julio Sosa</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.discogs.com/JGlQq8Q4mFy5ZdAmZrm52sAPV7S3gqKvmhCAfkyeJac/rs:fit/g:sm/q:40/h:300/w:300/czM6Ly9kaXNjb2dz/LWRhdGFiYXNlLWlt/YWdlcy9SLTk3ODI5/MzItMTYwNTU4NDg4/OC0zNDk2LmpwZWc.jpeg</t>
+    </r>
+  </si>
+  <si>
+    <t>Sting</t>
+  </si>
+  <si>
+    <t>The dream of the blue turtles</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273804c1bb88d714079e12d80e1</t>
+    </r>
+  </si>
+  <si>
+    <t>Tan Biónica</t>
+  </si>
+  <si>
+    <t>Hola Mundo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2730cef6c8d0af7bde036793c4a</t>
+    </r>
+  </si>
+  <si>
+    <t>Tipitos Los</t>
+  </si>
+  <si>
+    <t>Armando Camaleón</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2739934f74a9f25f2d4d0d9509e</t>
     </r>
   </si>
 </sst>
@@ -417,7 +894,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -431,9 +908,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1484,7 +1958,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="16.3516" style="1" customWidth="1"/>
@@ -1702,19 +2176,334 @@
       </c>
     </row>
     <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" s="5"/>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-    </row>
-    <row r="21" ht="20.05" customHeight="1">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5"/>
-      <c r="C21" s="5"/>
-    </row>
-    <row r="22" ht="20.05" customHeight="1">
-      <c r="A22" s="5"/>
-      <c r="B22" s="5"/>
-      <c r="C22" s="5"/>
+      <c r="A20" t="s" s="4">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s" s="4">
+        <v>53</v>
+      </c>
+      <c r="C20" t="s" s="4">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="21" ht="32.05" customHeight="1">
+      <c r="A21" t="s" s="4">
+        <v>55</v>
+      </c>
+      <c r="B21" t="s" s="4">
+        <v>56</v>
+      </c>
+      <c r="C21" t="s" s="4">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22" ht="32.05" customHeight="1">
+      <c r="A22" t="s" s="4">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s" s="4">
+        <v>59</v>
+      </c>
+      <c r="C22" t="s" s="4">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23" ht="20.05" customHeight="1">
+      <c r="A23" t="s" s="4">
+        <v>61</v>
+      </c>
+      <c r="B23" t="s" s="4">
+        <v>62</v>
+      </c>
+      <c r="C23" t="s" s="4">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" ht="44.05" customHeight="1">
+      <c r="A24" t="s" s="4">
+        <v>64</v>
+      </c>
+      <c r="B24" t="s" s="4">
+        <v>65</v>
+      </c>
+      <c r="C24" t="s" s="4">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" ht="20.05" customHeight="1">
+      <c r="A25" t="s" s="4">
+        <v>67</v>
+      </c>
+      <c r="B25" t="s" s="4">
+        <v>68</v>
+      </c>
+      <c r="C25" t="s" s="4">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" ht="20.05" customHeight="1">
+      <c r="A26" t="s" s="4">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s" s="4">
+        <v>71</v>
+      </c>
+      <c r="C26" t="s" s="4">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" ht="20.05" customHeight="1">
+      <c r="A27" t="s" s="4">
+        <v>70</v>
+      </c>
+      <c r="B27" t="s" s="4">
+        <v>73</v>
+      </c>
+      <c r="C27" t="s" s="4">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" ht="32.05" customHeight="1">
+      <c r="A28" t="s" s="4">
+        <v>75</v>
+      </c>
+      <c r="B28" t="s" s="4">
+        <v>76</v>
+      </c>
+      <c r="C28" t="s" s="4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="29" ht="32.05" customHeight="1">
+      <c r="A29" t="s" s="4">
+        <v>78</v>
+      </c>
+      <c r="B29" t="s" s="4">
+        <v>79</v>
+      </c>
+      <c r="C29" t="s" s="4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" ht="32.05" customHeight="1">
+      <c r="A30" t="s" s="4">
+        <v>81</v>
+      </c>
+      <c r="B30" t="s" s="4">
+        <v>82</v>
+      </c>
+      <c r="C30" t="s" s="4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" ht="20.05" customHeight="1">
+      <c r="A31" t="s" s="4">
+        <v>81</v>
+      </c>
+      <c r="B31" t="s" s="4">
+        <v>84</v>
+      </c>
+      <c r="C31" t="s" s="4">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="32" ht="20.05" customHeight="1">
+      <c r="A32" t="s" s="4">
+        <v>86</v>
+      </c>
+      <c r="B32" t="s" s="4">
+        <v>87</v>
+      </c>
+      <c r="C32" t="s" s="4">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="33" ht="20.05" customHeight="1">
+      <c r="A33" t="s" s="4">
+        <v>89</v>
+      </c>
+      <c r="B33" t="s" s="4">
+        <v>89</v>
+      </c>
+      <c r="C33" t="s" s="4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="34" ht="20.05" customHeight="1">
+      <c r="A34" t="s" s="4">
+        <v>89</v>
+      </c>
+      <c r="B34" t="s" s="4">
+        <v>91</v>
+      </c>
+      <c r="C34" t="s" s="4">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="35" ht="32.05" customHeight="1">
+      <c r="A35" t="s" s="4">
+        <v>89</v>
+      </c>
+      <c r="B35" t="s" s="4">
+        <v>93</v>
+      </c>
+      <c r="C35" t="s" s="4">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" ht="20.05" customHeight="1">
+      <c r="A36" t="s" s="4">
+        <v>89</v>
+      </c>
+      <c r="B36" t="s" s="4">
+        <v>95</v>
+      </c>
+      <c r="C36" t="s" s="4">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" ht="20.05" customHeight="1">
+      <c r="A37" t="s" s="4">
+        <v>97</v>
+      </c>
+      <c r="B37" t="s" s="4">
+        <v>97</v>
+      </c>
+      <c r="C37" t="s" s="4">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" ht="20.05" customHeight="1">
+      <c r="A38" t="s" s="4">
+        <v>99</v>
+      </c>
+      <c r="B38" t="s" s="4">
+        <v>100</v>
+      </c>
+      <c r="C38" t="s" s="4">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="39" ht="20.05" customHeight="1">
+      <c r="A39" t="s" s="4">
+        <v>99</v>
+      </c>
+      <c r="B39" t="s" s="4">
+        <v>102</v>
+      </c>
+      <c r="C39" t="s" s="4">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="40" ht="20.05" customHeight="1">
+      <c r="A40" t="s" s="4">
+        <v>104</v>
+      </c>
+      <c r="B40" t="s" s="4">
+        <v>105</v>
+      </c>
+      <c r="C40" t="s" s="4">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="41" ht="32.05" customHeight="1">
+      <c r="A41" t="s" s="4">
+        <v>107</v>
+      </c>
+      <c r="B41" t="s" s="4">
+        <v>108</v>
+      </c>
+      <c r="C41" t="s" s="4">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" ht="20.05" customHeight="1">
+      <c r="A42" t="s" s="4">
+        <v>110</v>
+      </c>
+      <c r="B42" t="s" s="4">
+        <v>111</v>
+      </c>
+      <c r="C42" t="s" s="4">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="43" ht="20.05" customHeight="1">
+      <c r="A43" t="s" s="4">
+        <v>110</v>
+      </c>
+      <c r="B43" t="s" s="4">
+        <v>113</v>
+      </c>
+      <c r="C43" t="s" s="4">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="44" ht="20.05" customHeight="1">
+      <c r="A44" t="s" s="4">
+        <v>110</v>
+      </c>
+      <c r="B44" t="s" s="4">
+        <v>115</v>
+      </c>
+      <c r="C44" t="s" s="4">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="45" ht="20.05" customHeight="1">
+      <c r="A45" t="s" s="4">
+        <v>110</v>
+      </c>
+      <c r="B45" t="s" s="4">
+        <v>117</v>
+      </c>
+      <c r="C45" t="s" s="4">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46" ht="32.05" customHeight="1">
+      <c r="A46" t="s" s="4">
+        <v>119</v>
+      </c>
+      <c r="B46" t="s" s="4">
+        <v>120</v>
+      </c>
+      <c r="C46" t="s" s="4">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="47" ht="32.05" customHeight="1">
+      <c r="A47" t="s" s="4">
+        <v>122</v>
+      </c>
+      <c r="B47" t="s" s="4">
+        <v>123</v>
+      </c>
+      <c r="C47" t="s" s="4">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" ht="20.05" customHeight="1">
+      <c r="A48" t="s" s="4">
+        <v>125</v>
+      </c>
+      <c r="B48" t="s" s="4">
+        <v>126</v>
+      </c>
+      <c r="C48" t="s" s="4">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="49" ht="20.05" customHeight="1">
+      <c r="A49" t="s" s="4">
+        <v>128</v>
+      </c>
+      <c r="B49" t="s" s="4">
+        <v>129</v>
+      </c>
+      <c r="C49" t="s" s="4">
+        <v>130</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -1736,6 +2525,36 @@
     <hyperlink ref="C17" r:id="rId16" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733e030a7e606959674643d274"/>
     <hyperlink ref="C18" r:id="rId17" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80"/>
     <hyperlink ref="C19" r:id="rId18" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b"/>
+    <hyperlink ref="C20" r:id="rId19" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279"/>
+    <hyperlink ref="C21" r:id="rId20" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7"/>
+    <hyperlink ref="C22" r:id="rId21" location="" tooltip="" display="https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg"/>
+    <hyperlink ref="C23" r:id="rId22" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473"/>
+    <hyperlink ref="C24" r:id="rId23" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4"/>
+    <hyperlink ref="C25" r:id="rId24" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f"/>
+    <hyperlink ref="C26" r:id="rId25" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff"/>
+    <hyperlink ref="C27" r:id="rId26" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca"/>
+    <hyperlink ref="C28" r:id="rId27" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e"/>
+    <hyperlink ref="C29" r:id="rId28" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400"/>
+    <hyperlink ref="C30" r:id="rId29" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08"/>
+    <hyperlink ref="C31" r:id="rId30" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3"/>
+    <hyperlink ref="C32" r:id="rId31" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135"/>
+    <hyperlink ref="C33" r:id="rId32" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87"/>
+    <hyperlink ref="C34" r:id="rId33" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419"/>
+    <hyperlink ref="C35" r:id="rId34" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537"/>
+    <hyperlink ref="C36" r:id="rId35" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02"/>
+    <hyperlink ref="C37" r:id="rId36" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733935c39bea149ac15c83c41a"/>
+    <hyperlink ref="C38" r:id="rId37" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730320739a960dd4821b2aeaf1"/>
+    <hyperlink ref="C39" r:id="rId38" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273139d10e0ae979a7b4a811140"/>
+    <hyperlink ref="C40" r:id="rId39" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733443d9c76e9713a5986c983c"/>
+    <hyperlink ref="C41" r:id="rId40" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dfc72dec3da479c81c575551"/>
+    <hyperlink ref="C42" r:id="rId41" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c3780b28120b1bc2869a2ca7"/>
+    <hyperlink ref="C43" r:id="rId42" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737e553e1367924fa3429a692c"/>
+    <hyperlink ref="C44" r:id="rId43" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e28947f6ad2f100af9c1965a"/>
+    <hyperlink ref="C45" r:id="rId44" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273d8abc667a17dab2e1a6bd44e"/>
+    <hyperlink ref="C46" r:id="rId45" location="" tooltip="" display="https://i.discogs.com/JGlQq8Q4mFy5ZdAmZrm52sAPV7S3gqKvmhCAfkyeJac/rs:fit/g:sm/q:40/h:300/w:300/czM6Ly9kaXNjb2dz/LWRhdGFiYXNlLWlt/YWdlcy9SLTk3ODI5/MzItMTYwNTU4NDg4/OC0zNDk2LmpwZWc.jpeg"/>
+    <hyperlink ref="C47" r:id="rId46" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273804c1bb88d714079e12d80e1"/>
+    <hyperlink ref="C48" r:id="rId47" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730cef6c8d0af7bde036793c4a"/>
+    <hyperlink ref="C49" r:id="rId48" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739934f74a9f25f2d4d0d9509e"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
Actualizo 22 2 26
</commit_message>
<xml_diff>
--- a/public/discos.xlsx
+++ b/public/discos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="162">
   <si>
     <t>Artista</t>
   </si>
@@ -22,6 +22,23 @@
     <t>Imagen</t>
   </si>
   <si>
+    <t>A-ha</t>
+  </si>
+  <si>
+    <t>Hunting high and low</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e8dd4db47e7177c63b0b7d53</t>
+    </r>
+  </si>
+  <si>
     <t>ABBA</t>
   </si>
   <si>
@@ -39,23 +56,6 @@
     </r>
   </si>
   <si>
-    <t>A-ha</t>
-  </si>
-  <si>
-    <t>Hunting high and low</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273e8dd4db47e7177c63b0b7d53</t>
-    </r>
-  </si>
-  <si>
     <t>Almendra</t>
   </si>
   <si>
@@ -70,6 +70,37 @@
     </r>
   </si>
   <si>
+    <t>Arctic Monkeys</t>
+  </si>
+  <si>
+    <t>AM</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2734ae1c4c5c45aabe565499163</t>
+    </r>
+  </si>
+  <si>
+    <t>Tranquility Base Hotel &amp; Casino</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2738895ff0f90525f4aa9437c27</t>
+    </r>
+  </si>
+  <si>
     <t>Beatles The</t>
   </si>
   <si>
@@ -152,6 +183,48 @@
     </r>
   </si>
   <si>
+    <t>Amor Amarillo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885</t>
+    </r>
+  </si>
+  <si>
+    <t>Bocanada</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab</t>
+    </r>
+  </si>
+  <si>
+    <t>Siempre es Hoy</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27392441ecd34874c2bc4f19144</t>
+    </r>
+  </si>
+  <si>
     <t>Coldplay</t>
   </si>
   <si>
@@ -169,6 +242,20 @@
     </r>
   </si>
   <si>
+    <t>Viva la Vida</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e21cc1db05580b6f2d2a3b6e</t>
+    </r>
+  </si>
+  <si>
     <t>Conociendo Rusia</t>
   </si>
   <si>
@@ -200,6 +287,40 @@
     </r>
   </si>
   <si>
+    <t>Daft Punk</t>
+  </si>
+  <si>
+    <t>Random Access Memory</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2739b9b36b0e22870b9f542d937</t>
+    </r>
+  </si>
+  <si>
+    <t>David Guetta</t>
+  </si>
+  <si>
+    <t>Nothing but the beat</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7</t>
+    </r>
+  </si>
+  <si>
     <t>Deep Purple</t>
   </si>
   <si>
@@ -265,6 +386,23 @@
     </r>
   </si>
   <si>
+    <t>Fito Paez</t>
+  </si>
+  <si>
+    <t>Giros</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80</t>
+    </r>
+  </si>
+  <si>
     <t>Foreigner</t>
   </si>
   <si>
@@ -282,23 +420,6 @@
     </r>
   </si>
   <si>
-    <t>Fito Paez</t>
-  </si>
-  <si>
-    <t>Giros</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80</t>
-    </r>
-  </si>
-  <si>
     <t>Gorillaz</t>
   </si>
   <si>
@@ -330,23 +451,6 @@
     </r>
   </si>
   <si>
-    <t>David Guetta</t>
-  </si>
-  <si>
-    <t>Nothing but the beat</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7</t>
-    </r>
-  </si>
-  <si>
     <t>Harrison George</t>
   </si>
   <si>
@@ -528,6 +632,40 @@
     </r>
   </si>
   <si>
+    <t>Pescado Rabioso</t>
+  </si>
+  <si>
+    <t>Artaud</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27350db5a166ea23d5d6c4cd387</t>
+    </r>
+  </si>
+  <si>
+    <t>Pointed Sisters</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273ef221258ca5f3e223937d408</t>
+    </r>
+  </si>
+  <si>
     <t>Queen</t>
   </si>
   <si>
@@ -584,6 +722,48 @@
     </r>
   </si>
   <si>
+    <t>A day at the Races</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492</t>
+    </r>
+  </si>
+  <si>
+    <t>Queen II</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273b57713d0fe3553a087419f8f</t>
+    </r>
+  </si>
+  <si>
+    <t>The Game</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273056e90910cbaf5c5b892aeba</t>
+    </r>
+  </si>
+  <si>
     <t>Ramones</t>
   </si>
   <si>
@@ -643,6 +823,23 @@
         <rFont val="Helvetica Neue"/>
       </rPr>
       <t>https://i.scdn.co/image/ab67616d0000b2733443d9c76e9713a5986c983c</t>
+    </r>
+  </si>
+  <si>
+    <t>Seru Giran</t>
+  </si>
+  <si>
+    <t>Serú 92</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273ac84ce59dc5d49c81dc9d8fb</t>
     </r>
   </si>
   <si>
@@ -797,7 +994,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -807,6 +1004,11 @@
       <sz val="12"/>
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
+    </font>
+    <font>
+      <sz val="15"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b val="1"/>
@@ -820,8 +1022,14 @@
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
     </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color indexed="14"/>
+      <name val="Helvetica Neue"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -834,8 +1042,14 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="11"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -854,7 +1068,7 @@
         <color indexed="10"/>
       </top>
       <bottom style="thin">
-        <color indexed="11"/>
+        <color indexed="10"/>
       </bottom>
       <diagonal/>
     </border>
@@ -862,15 +1076,22 @@
       <left style="thin">
         <color indexed="10"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color indexed="12"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
-        <color indexed="10"/>
+        <color indexed="12"/>
       </right>
       <top style="thin">
-        <color indexed="11"/>
+        <color indexed="12"/>
       </top>
-      <bottom style="thin">
-        <color indexed="10"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -884,7 +1105,62 @@
         <color indexed="10"/>
       </top>
       <bottom style="thin">
+        <color indexed="13"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color indexed="10"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right style="thin">
+        <color indexed="10"/>
+      </right>
+      <top style="thin">
+        <color indexed="13"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="10"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="10"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="12"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="12"/>
       </bottom>
       <diagonal/>
     </border>
@@ -894,21 +1170,42 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -929,7 +1226,10 @@
       <rgbColor rgb="ff000000"/>
       <rgbColor rgb="ffbdc0bf"/>
       <rgbColor rgb="ffa5a5a5"/>
+      <rgbColor rgb="ffffffff"/>
+      <rgbColor rgb="ffaaaaaa"/>
       <rgbColor rgb="ff3f3f3f"/>
+      <rgbColor rgb="ff0000ff"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -946,10 +1246,10 @@
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="5E5E5E"/>
+        <a:srgbClr val="A7A7A7"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="D5D5D5"/>
+        <a:srgbClr val="535353"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="00A2FF"/>
@@ -1126,11 +1426,14 @@
     <a:spDef>
       <a:spPr>
         <a:solidFill>
-          <a:srgbClr val="000000"/>
+          <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
+        <a:ln w="25400" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1139,7 +1442,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="ctr" defTabSz="584200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1153,19 +1456,19 @@
           <a:buSzTx/>
           <a:buFontTx/>
           <a:buNone/>
-          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1200" u="none" kumimoji="0" normalizeH="0">
+          <a:defRPr b="0" baseline="0" cap="none" i="0" spc="0" strike="noStrike" sz="1100" u="none" kumimoji="0" normalizeH="0">
             <a:ln>
               <a:noFill/>
             </a:ln>
             <a:solidFill>
-              <a:srgbClr val="FFFFFF"/>
+              <a:srgbClr val="000000"/>
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Helvetica Neue Medium"/>
-            <a:ea typeface="Helvetica Neue Medium"/>
-            <a:cs typeface="Helvetica Neue Medium"/>
-            <a:sym typeface="Helvetica Neue Medium"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1404,12 +1707,12 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="12700" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
-            <a:srgbClr val="000000"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="400000"/>
+          <a:round/>
         </a:ln>
         <a:effectLst/>
         <a:sp3d/>
@@ -1690,7 +1993,7 @@
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
-        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="457200" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
+        <a:defPPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="0" hangingPunct="0">
           <a:lnSpc>
             <a:spcPct val="100000"/>
           </a:lnSpc>
@@ -1958,12 +2261,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="19.9" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="2" width="16.3516" style="1" customWidth="1"/>
-    <col min="3" max="3" width="104.094" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="16.3516" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.3516" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.6328" style="1" customWidth="1"/>
+    <col min="3" max="3" width="104.172" style="1" customWidth="1"/>
+    <col min="4" max="5" width="16.3516" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.25" customHeight="1">
@@ -1976,585 +2281,865 @@
       <c r="C1" t="s" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" ht="32.25" customHeight="1">
-      <c r="A2" t="s" s="3">
+      <c r="D1" s="3"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" ht="32.05" customHeight="1">
+      <c r="A2" t="s" s="5">
         <v>3</v>
       </c>
-      <c r="B2" t="s" s="3">
+      <c r="B2" t="s" s="5">
         <v>4</v>
       </c>
-      <c r="C2" t="s" s="3">
+      <c r="C2" t="s" s="5">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" ht="32.05" customHeight="1">
-      <c r="A3" t="s" s="4">
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+    </row>
+    <row r="3" ht="32.25" customHeight="1">
+      <c r="A3" t="s" s="8">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="4">
+      <c r="B3" t="s" s="8">
         <v>7</v>
       </c>
-      <c r="C3" t="s" s="4">
+      <c r="C3" t="s" s="8">
         <v>8</v>
       </c>
+      <c r="D3" s="6"/>
+      <c r="E3" s="7"/>
     </row>
     <row r="4" ht="20.05" customHeight="1">
-      <c r="A4" t="s" s="4">
+      <c r="A4" t="s" s="9">
         <v>9</v>
       </c>
-      <c r="B4" t="s" s="4">
+      <c r="B4" t="s" s="9">
         <v>9</v>
       </c>
-      <c r="C4" t="s" s="4">
+      <c r="C4" t="s" s="9">
         <v>10</v>
       </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" ht="20.05" customHeight="1">
-      <c r="A5" t="s" s="4">
+      <c r="A5" t="s" s="9">
         <v>11</v>
       </c>
-      <c r="B5" t="s" s="4">
+      <c r="B5" t="s" s="9">
         <v>12</v>
       </c>
-      <c r="C5" t="s" s="4">
+      <c r="C5" t="s" s="9">
         <v>13</v>
       </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="7"/>
     </row>
     <row r="6" ht="20.05" customHeight="1">
-      <c r="A6" t="s" s="4">
+      <c r="A6" t="s" s="9">
         <v>11</v>
       </c>
-      <c r="B6" t="s" s="4">
+      <c r="B6" t="s" s="9">
         <v>14</v>
       </c>
-      <c r="C6" t="s" s="4">
+      <c r="C6" t="s" s="9">
         <v>15</v>
       </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="7"/>
     </row>
     <row r="7" ht="20.05" customHeight="1">
-      <c r="A7" t="s" s="4">
+      <c r="A7" t="s" s="9">
         <v>16</v>
       </c>
-      <c r="B7" t="s" s="4">
+      <c r="B7" t="s" s="9">
         <v>17</v>
       </c>
-      <c r="C7" t="s" s="4">
+      <c r="C7" t="s" s="9">
         <v>18</v>
       </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="7"/>
     </row>
     <row r="8" ht="20.05" customHeight="1">
-      <c r="A8" t="s" s="4">
+      <c r="A8" t="s" s="9">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s" s="9">
         <v>19</v>
       </c>
-      <c r="B8" t="s" s="4">
+      <c r="C8" t="s" s="9">
         <v>20</v>
       </c>
-      <c r="C8" t="s" s="4">
+      <c r="D8" s="6"/>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="9" ht="20.05" customHeight="1">
+      <c r="A9" t="s" s="9">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" ht="20.05" customHeight="1">
-      <c r="A9" t="s" s="4">
+      <c r="B9" t="s" s="9">
         <v>22</v>
       </c>
-      <c r="B9" t="s" s="4">
+      <c r="C9" t="s" s="9">
         <v>23</v>
       </c>
-      <c r="C9" t="s" s="4">
+      <c r="D9" s="6"/>
+      <c r="E9" s="7"/>
+    </row>
+    <row r="10" ht="20.05" customHeight="1">
+      <c r="A10" t="s" s="9">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" ht="20.05" customHeight="1">
-      <c r="A10" t="s" s="4">
+      <c r="B10" t="s" s="9">
         <v>25</v>
       </c>
-      <c r="B10" t="s" s="4">
+      <c r="C10" t="s" s="9">
         <v>26</v>
       </c>
-      <c r="C10" t="s" s="4">
+      <c r="D10" s="6"/>
+      <c r="E10" s="7"/>
+    </row>
+    <row r="11" ht="20.05" customHeight="1">
+      <c r="A11" t="s" s="9">
         <v>27</v>
       </c>
-    </row>
-    <row r="11" ht="32.05" customHeight="1">
-      <c r="A11" t="s" s="4">
+      <c r="B11" t="s" s="9">
         <v>28</v>
       </c>
-      <c r="B11" t="s" s="4">
+      <c r="C11" t="s" s="9">
         <v>29</v>
       </c>
-      <c r="C11" t="s" s="4">
+      <c r="D11" s="6"/>
+      <c r="E11" s="7"/>
+    </row>
+    <row r="12" ht="20.05" customHeight="1">
+      <c r="A12" t="s" s="9">
+        <v>27</v>
+      </c>
+      <c r="B12" t="s" s="9">
         <v>30</v>
       </c>
-    </row>
-    <row r="12" ht="20.05" customHeight="1">
-      <c r="A12" t="s" s="4">
-        <v>28</v>
-      </c>
-      <c r="B12" t="s" s="4">
+      <c r="C12" t="s" s="9">
         <v>31</v>
       </c>
-      <c r="C12" t="s" s="4">
+      <c r="D12" s="6"/>
+      <c r="E12" s="7"/>
+    </row>
+    <row r="13" ht="20.05" customHeight="1">
+      <c r="A13" t="s" s="9">
+        <v>27</v>
+      </c>
+      <c r="B13" t="s" s="9">
         <v>32</v>
       </c>
-    </row>
-    <row r="13" ht="20.05" customHeight="1">
-      <c r="A13" t="s" s="4">
+      <c r="C13" t="s" s="9">
         <v>33</v>
       </c>
-      <c r="B13" t="s" s="4">
+      <c r="D13" s="6"/>
+      <c r="E13" s="7"/>
+    </row>
+    <row r="14" ht="20.05" customHeight="1">
+      <c r="A14" t="s" s="9">
+        <v>27</v>
+      </c>
+      <c r="B14" t="s" s="9">
         <v>34</v>
       </c>
-      <c r="C13" t="s" s="4">
+      <c r="C14" t="s" s="9">
         <v>35</v>
       </c>
-    </row>
-    <row r="14" ht="20.05" customHeight="1">
-      <c r="A14" t="s" s="4">
+      <c r="D14" s="6"/>
+      <c r="E14" s="7"/>
+    </row>
+    <row r="15" ht="20.05" customHeight="1">
+      <c r="A15" t="s" s="9">
         <v>36</v>
       </c>
-      <c r="B14" t="s" s="4">
+      <c r="B15" t="s" s="9">
         <v>37</v>
       </c>
-      <c r="C14" t="s" s="4">
+      <c r="C15" t="s" s="9">
         <v>38</v>
       </c>
-    </row>
-    <row r="15" ht="20.05" customHeight="1">
-      <c r="A15" t="s" s="4">
+      <c r="D15" s="6"/>
+      <c r="E15" s="7"/>
+    </row>
+    <row r="16" ht="20.05" customHeight="1">
+      <c r="A16" t="s" s="9">
+        <v>36</v>
+      </c>
+      <c r="B16" t="s" s="9">
         <v>39</v>
       </c>
-      <c r="B15" t="s" s="4">
+      <c r="C16" t="s" s="9">
         <v>40</v>
       </c>
-      <c r="C15" t="s" s="4">
+      <c r="D16" s="6"/>
+      <c r="E16" s="7"/>
+    </row>
+    <row r="17" ht="32.05" customHeight="1">
+      <c r="A17" t="s" s="9">
         <v>41</v>
       </c>
-    </row>
-    <row r="16" ht="20.05" customHeight="1">
-      <c r="A16" t="s" s="4">
-        <v>39</v>
-      </c>
-      <c r="B16" t="s" s="4">
+      <c r="B17" t="s" s="9">
         <v>42</v>
       </c>
-      <c r="C16" t="s" s="4">
+      <c r="C17" t="s" s="9">
         <v>43</v>
       </c>
-    </row>
-    <row r="17" ht="20.05" customHeight="1">
-      <c r="A17" t="s" s="4">
+      <c r="D17" s="6"/>
+      <c r="E17" s="7"/>
+    </row>
+    <row r="18" ht="20.05" customHeight="1">
+      <c r="A18" t="s" s="9">
+        <v>41</v>
+      </c>
+      <c r="B18" t="s" s="9">
         <v>44</v>
       </c>
-      <c r="B17" t="s" s="4">
+      <c r="C18" t="s" s="9">
         <v>45</v>
       </c>
-      <c r="C17" t="s" s="4">
+      <c r="D18" s="6"/>
+      <c r="E18" s="7"/>
+    </row>
+    <row r="19" ht="20.05" customHeight="1">
+      <c r="A19" t="s" s="9">
         <v>46</v>
       </c>
-    </row>
-    <row r="18" ht="20.05" customHeight="1">
-      <c r="A18" t="s" s="4">
+      <c r="B19" t="s" s="9">
         <v>47</v>
       </c>
-      <c r="B18" t="s" s="4">
+      <c r="C19" t="s" s="9">
         <v>48</v>
       </c>
-      <c r="C18" t="s" s="4">
+      <c r="D19" s="6"/>
+      <c r="E19" s="7"/>
+    </row>
+    <row r="20" ht="32.05" customHeight="1">
+      <c r="A20" t="s" s="9">
         <v>49</v>
       </c>
-    </row>
-    <row r="19" ht="20.05" customHeight="1">
-      <c r="A19" t="s" s="4">
+      <c r="B20" t="s" s="9">
         <v>50</v>
       </c>
-      <c r="B19" t="s" s="4">
-        <v>50</v>
-      </c>
-      <c r="C19" t="s" s="4">
+      <c r="C20" t="s" s="9">
         <v>51</v>
       </c>
-    </row>
-    <row r="20" ht="20.05" customHeight="1">
-      <c r="A20" t="s" s="4">
+      <c r="D20" s="6"/>
+      <c r="E20" s="7"/>
+    </row>
+    <row r="21" ht="20.05" customHeight="1">
+      <c r="A21" t="s" s="9">
         <v>52</v>
       </c>
-      <c r="B20" t="s" s="4">
+      <c r="B21" t="s" s="9">
         <v>53</v>
       </c>
-      <c r="C20" t="s" s="4">
+      <c r="C21" t="s" s="9">
         <v>54</v>
       </c>
-    </row>
-    <row r="21" ht="32.05" customHeight="1">
-      <c r="A21" t="s" s="4">
+      <c r="D21" s="6"/>
+      <c r="E21" s="7"/>
+    </row>
+    <row r="22" ht="20.05" customHeight="1">
+      <c r="A22" t="s" s="9">
         <v>55</v>
       </c>
-      <c r="B21" t="s" s="4">
+      <c r="B22" t="s" s="9">
         <v>56</v>
       </c>
-      <c r="C21" t="s" s="4">
+      <c r="C22" t="s" s="9">
         <v>57</v>
       </c>
-    </row>
-    <row r="22" ht="32.05" customHeight="1">
-      <c r="A22" t="s" s="4">
+      <c r="D22" s="6"/>
+      <c r="E22" s="7"/>
+    </row>
+    <row r="23" ht="20.05" customHeight="1">
+      <c r="A23" t="s" s="9">
         <v>58</v>
       </c>
-      <c r="B22" t="s" s="4">
+      <c r="B23" t="s" s="9">
         <v>59</v>
       </c>
-      <c r="C22" t="s" s="4">
+      <c r="C23" t="s" s="9">
         <v>60</v>
       </c>
-    </row>
-    <row r="23" ht="20.05" customHeight="1">
-      <c r="A23" t="s" s="4">
+      <c r="D23" s="6"/>
+      <c r="E23" s="7"/>
+    </row>
+    <row r="24" ht="20.05" customHeight="1">
+      <c r="A24" t="s" s="9">
+        <v>58</v>
+      </c>
+      <c r="B24" t="s" s="9">
         <v>61</v>
       </c>
-      <c r="B23" t="s" s="4">
+      <c r="C24" t="s" s="9">
         <v>62</v>
       </c>
-      <c r="C23" t="s" s="4">
+      <c r="D24" s="6"/>
+      <c r="E24" s="7"/>
+    </row>
+    <row r="25" ht="20.05" customHeight="1">
+      <c r="A25" t="s" s="9">
         <v>63</v>
       </c>
-    </row>
-    <row r="24" ht="44.05" customHeight="1">
-      <c r="A24" t="s" s="4">
+      <c r="B25" t="s" s="9">
         <v>64</v>
       </c>
-      <c r="B24" t="s" s="4">
+      <c r="C25" t="s" s="9">
         <v>65</v>
       </c>
-      <c r="C24" t="s" s="4">
+      <c r="D25" s="6"/>
+      <c r="E25" s="7"/>
+    </row>
+    <row r="26" ht="20.05" customHeight="1">
+      <c r="A26" t="s" s="9">
         <v>66</v>
       </c>
-    </row>
-    <row r="25" ht="20.05" customHeight="1">
-      <c r="A25" t="s" s="4">
+      <c r="B26" t="s" s="9">
         <v>67</v>
       </c>
-      <c r="B25" t="s" s="4">
+      <c r="C26" t="s" s="9">
         <v>68</v>
       </c>
-      <c r="C25" t="s" s="4">
+      <c r="D26" s="6"/>
+      <c r="E26" s="7"/>
+    </row>
+    <row r="27" ht="20.05" customHeight="1">
+      <c r="A27" t="s" s="9">
         <v>69</v>
       </c>
-    </row>
-    <row r="26" ht="20.05" customHeight="1">
-      <c r="A26" t="s" s="4">
+      <c r="B27" t="s" s="9">
+        <v>69</v>
+      </c>
+      <c r="C27" t="s" s="9">
         <v>70</v>
       </c>
-      <c r="B26" t="s" s="4">
+      <c r="D27" s="6"/>
+      <c r="E27" s="7"/>
+    </row>
+    <row r="28" ht="20.05" customHeight="1">
+      <c r="A28" t="s" s="9">
         <v>71</v>
       </c>
-      <c r="C26" t="s" s="4">
+      <c r="B28" t="s" s="9">
         <v>72</v>
       </c>
-    </row>
-    <row r="27" ht="20.05" customHeight="1">
-      <c r="A27" t="s" s="4">
-        <v>70</v>
-      </c>
-      <c r="B27" t="s" s="4">
+      <c r="C28" t="s" s="9">
         <v>73</v>
       </c>
-      <c r="C27" t="s" s="4">
+      <c r="D28" s="6"/>
+      <c r="E28" s="7"/>
+    </row>
+    <row r="29" ht="32.05" customHeight="1">
+      <c r="A29" t="s" s="9">
         <v>74</v>
       </c>
-    </row>
-    <row r="28" ht="32.05" customHeight="1">
-      <c r="A28" t="s" s="4">
+      <c r="B29" t="s" s="9">
         <v>75</v>
       </c>
-      <c r="B28" t="s" s="4">
+      <c r="C29" t="s" s="9">
         <v>76</v>
       </c>
-      <c r="C28" t="s" s="4">
+      <c r="D29" s="6"/>
+      <c r="E29" s="7"/>
+    </row>
+    <row r="30" ht="20.05" customHeight="1">
+      <c r="A30" t="s" s="9">
         <v>77</v>
       </c>
-    </row>
-    <row r="29" ht="32.05" customHeight="1">
-      <c r="A29" t="s" s="4">
+      <c r="B30" t="s" s="9">
         <v>78</v>
       </c>
-      <c r="B29" t="s" s="4">
+      <c r="C30" t="s" s="9">
         <v>79</v>
       </c>
-      <c r="C29" t="s" s="4">
+      <c r="D30" s="6"/>
+      <c r="E30" s="7"/>
+    </row>
+    <row r="31" ht="44.05" customHeight="1">
+      <c r="A31" t="s" s="9">
         <v>80</v>
       </c>
-    </row>
-    <row r="30" ht="32.05" customHeight="1">
-      <c r="A30" t="s" s="4">
+      <c r="B31" t="s" s="9">
         <v>81</v>
       </c>
-      <c r="B30" t="s" s="4">
+      <c r="C31" t="s" s="9">
         <v>82</v>
       </c>
-      <c r="C30" t="s" s="4">
+      <c r="D31" s="6"/>
+      <c r="E31" s="7"/>
+    </row>
+    <row r="32" ht="20.05" customHeight="1">
+      <c r="A32" t="s" s="9">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" ht="20.05" customHeight="1">
-      <c r="A31" t="s" s="4">
-        <v>81</v>
-      </c>
-      <c r="B31" t="s" s="4">
+      <c r="B32" t="s" s="9">
         <v>84</v>
       </c>
-      <c r="C31" t="s" s="4">
+      <c r="C32" t="s" s="9">
         <v>85</v>
       </c>
-    </row>
-    <row r="32" ht="20.05" customHeight="1">
-      <c r="A32" t="s" s="4">
+      <c r="D32" s="6"/>
+      <c r="E32" s="7"/>
+    </row>
+    <row r="33" ht="20.05" customHeight="1">
+      <c r="A33" t="s" s="9">
         <v>86</v>
       </c>
-      <c r="B32" t="s" s="4">
+      <c r="B33" t="s" s="9">
         <v>87</v>
       </c>
-      <c r="C32" t="s" s="4">
+      <c r="C33" t="s" s="9">
         <v>88</v>
       </c>
-    </row>
-    <row r="33" ht="20.05" customHeight="1">
-      <c r="A33" t="s" s="4">
+      <c r="D33" s="6"/>
+      <c r="E33" s="7"/>
+    </row>
+    <row r="34" ht="20.05" customHeight="1">
+      <c r="A34" t="s" s="9">
+        <v>86</v>
+      </c>
+      <c r="B34" t="s" s="9">
         <v>89</v>
       </c>
-      <c r="B33" t="s" s="4">
-        <v>89</v>
-      </c>
-      <c r="C33" t="s" s="4">
+      <c r="C34" t="s" s="9">
         <v>90</v>
       </c>
-    </row>
-    <row r="34" ht="20.05" customHeight="1">
-      <c r="A34" t="s" s="4">
-        <v>89</v>
-      </c>
-      <c r="B34" t="s" s="4">
+      <c r="D34" s="6"/>
+      <c r="E34" s="7"/>
+    </row>
+    <row r="35" ht="32.05" customHeight="1">
+      <c r="A35" t="s" s="9">
         <v>91</v>
       </c>
-      <c r="C34" t="s" s="4">
+      <c r="B35" t="s" s="9">
         <v>92</v>
       </c>
-    </row>
-    <row r="35" ht="32.05" customHeight="1">
-      <c r="A35" t="s" s="4">
-        <v>89</v>
-      </c>
-      <c r="B35" t="s" s="4">
+      <c r="C35" t="s" s="9">
         <v>93</v>
       </c>
-      <c r="C35" t="s" s="4">
+      <c r="D35" s="6"/>
+      <c r="E35" s="7"/>
+    </row>
+    <row r="36" ht="32.05" customHeight="1">
+      <c r="A36" t="s" s="9">
         <v>94</v>
       </c>
-    </row>
-    <row r="36" ht="20.05" customHeight="1">
-      <c r="A36" t="s" s="4">
-        <v>89</v>
-      </c>
-      <c r="B36" t="s" s="4">
+      <c r="B36" t="s" s="9">
         <v>95</v>
       </c>
-      <c r="C36" t="s" s="4">
+      <c r="C36" t="s" s="9">
         <v>96</v>
       </c>
-    </row>
-    <row r="37" ht="20.05" customHeight="1">
-      <c r="A37" t="s" s="4">
+      <c r="D36" s="6"/>
+      <c r="E36" s="7"/>
+    </row>
+    <row r="37" ht="32.05" customHeight="1">
+      <c r="A37" t="s" s="9">
         <v>97</v>
       </c>
-      <c r="B37" t="s" s="4">
+      <c r="B37" t="s" s="9">
+        <v>98</v>
+      </c>
+      <c r="C37" t="s" s="9">
+        <v>99</v>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="7"/>
+    </row>
+    <row r="38" ht="20.05" customHeight="1">
+      <c r="A38" t="s" s="9">
         <v>97</v>
       </c>
-      <c r="C37" t="s" s="4">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" ht="20.05" customHeight="1">
-      <c r="A38" t="s" s="4">
-        <v>99</v>
-      </c>
-      <c r="B38" t="s" s="4">
+      <c r="B38" t="s" s="9">
         <v>100</v>
       </c>
-      <c r="C38" t="s" s="4">
+      <c r="C38" t="s" s="9">
         <v>101</v>
       </c>
+      <c r="D38" s="6"/>
+      <c r="E38" s="7"/>
     </row>
     <row r="39" ht="20.05" customHeight="1">
-      <c r="A39" t="s" s="4">
-        <v>99</v>
-      </c>
-      <c r="B39" t="s" s="4">
+      <c r="A39" t="s" s="9">
         <v>102</v>
       </c>
-      <c r="C39" t="s" s="4">
+      <c r="B39" t="s" s="9">
         <v>103</v>
       </c>
+      <c r="C39" t="s" s="9">
+        <v>104</v>
+      </c>
+      <c r="D39" s="6"/>
+      <c r="E39" s="7"/>
     </row>
     <row r="40" ht="20.05" customHeight="1">
-      <c r="A40" t="s" s="4">
-        <v>104</v>
-      </c>
-      <c r="B40" t="s" s="4">
+      <c r="A40" t="s" s="9">
         <v>105</v>
       </c>
-      <c r="C40" t="s" s="4">
+      <c r="B40" t="s" s="9">
         <v>106</v>
       </c>
-    </row>
-    <row r="41" ht="32.05" customHeight="1">
-      <c r="A41" t="s" s="4">
+      <c r="C40" t="s" s="9">
         <v>107</v>
       </c>
-      <c r="B41" t="s" s="4">
+      <c r="D40" s="6"/>
+      <c r="E40" s="7"/>
+    </row>
+    <row r="41" ht="20.05" customHeight="1">
+      <c r="A41" t="s" s="9">
         <v>108</v>
       </c>
-      <c r="C41" t="s" s="4">
+      <c r="B41" t="s" s="9">
         <v>109</v>
       </c>
+      <c r="C41" t="s" s="9">
+        <v>110</v>
+      </c>
+      <c r="D41" s="6"/>
+      <c r="E41" s="7"/>
     </row>
     <row r="42" ht="20.05" customHeight="1">
-      <c r="A42" t="s" s="4">
-        <v>110</v>
-      </c>
-      <c r="B42" t="s" s="4">
+      <c r="A42" t="s" s="9">
         <v>111</v>
       </c>
-      <c r="C42" t="s" s="4">
+      <c r="B42" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="C42" t="s" s="9">
         <v>112</v>
       </c>
+      <c r="D42" s="6"/>
+      <c r="E42" s="7"/>
     </row>
     <row r="43" ht="20.05" customHeight="1">
-      <c r="A43" t="s" s="4">
-        <v>110</v>
-      </c>
-      <c r="B43" t="s" s="4">
+      <c r="A43" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B43" t="s" s="9">
         <v>113</v>
       </c>
-      <c r="C43" t="s" s="4">
+      <c r="C43" t="s" s="9">
         <v>114</v>
       </c>
-    </row>
-    <row r="44" ht="20.05" customHeight="1">
-      <c r="A44" t="s" s="4">
-        <v>110</v>
-      </c>
-      <c r="B44" t="s" s="4">
+      <c r="D43" s="6"/>
+      <c r="E43" s="7"/>
+    </row>
+    <row r="44" ht="32.05" customHeight="1">
+      <c r="A44" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B44" t="s" s="9">
         <v>115</v>
       </c>
-      <c r="C44" t="s" s="4">
+      <c r="C44" t="s" s="9">
         <v>116</v>
       </c>
+      <c r="D44" s="6"/>
+      <c r="E44" s="7"/>
     </row>
     <row r="45" ht="20.05" customHeight="1">
-      <c r="A45" t="s" s="4">
-        <v>110</v>
-      </c>
-      <c r="B45" t="s" s="4">
+      <c r="A45" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B45" t="s" s="9">
         <v>117</v>
       </c>
-      <c r="C45" t="s" s="4">
+      <c r="C45" t="s" s="9">
         <v>118</v>
       </c>
-    </row>
-    <row r="46" ht="32.05" customHeight="1">
-      <c r="A46" t="s" s="4">
+      <c r="D45" s="6"/>
+      <c r="E45" s="7"/>
+    </row>
+    <row r="46" ht="20.05" customHeight="1">
+      <c r="A46" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B46" t="s" s="9">
         <v>119</v>
       </c>
-      <c r="B46" t="s" s="4">
+      <c r="C46" t="s" s="9">
         <v>120</v>
       </c>
-      <c r="C46" t="s" s="4">
+      <c r="D46" s="6"/>
+      <c r="E46" s="7"/>
+    </row>
+    <row r="47" ht="20.05" customHeight="1">
+      <c r="A47" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B47" t="s" s="9">
         <v>121</v>
       </c>
-    </row>
-    <row r="47" ht="32.05" customHeight="1">
-      <c r="A47" t="s" s="4">
+      <c r="C47" t="s" s="9">
         <v>122</v>
       </c>
-      <c r="B47" t="s" s="4">
+      <c r="D47" s="6"/>
+      <c r="E47" s="7"/>
+    </row>
+    <row r="48" ht="20.05" customHeight="1">
+      <c r="A48" t="s" s="9">
+        <v>111</v>
+      </c>
+      <c r="B48" t="s" s="9">
         <v>123</v>
       </c>
-      <c r="C47" t="s" s="4">
+      <c r="C48" t="s" s="9">
         <v>124</v>
       </c>
-    </row>
-    <row r="48" ht="20.05" customHeight="1">
-      <c r="A48" t="s" s="4">
+      <c r="D48" s="6"/>
+      <c r="E48" s="7"/>
+    </row>
+    <row r="49" ht="20.05" customHeight="1">
+      <c r="A49" t="s" s="9">
         <v>125</v>
       </c>
-      <c r="B48" t="s" s="4">
+      <c r="B49" t="s" s="9">
+        <v>125</v>
+      </c>
+      <c r="C49" t="s" s="9">
         <v>126</v>
       </c>
-      <c r="C48" t="s" s="4">
+      <c r="D49" s="6"/>
+      <c r="E49" s="7"/>
+    </row>
+    <row r="50" ht="20.05" customHeight="1">
+      <c r="A50" t="s" s="9">
         <v>127</v>
       </c>
-    </row>
-    <row r="49" ht="20.05" customHeight="1">
-      <c r="A49" t="s" s="4">
+      <c r="B50" t="s" s="9">
         <v>128</v>
       </c>
-      <c r="B49" t="s" s="4">
+      <c r="C50" t="s" s="9">
         <v>129</v>
       </c>
-      <c r="C49" t="s" s="4">
+      <c r="D50" s="6"/>
+      <c r="E50" s="7"/>
+    </row>
+    <row r="51" ht="20.05" customHeight="1">
+      <c r="A51" t="s" s="9">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s" s="9">
         <v>130</v>
       </c>
+      <c r="C51" t="s" s="9">
+        <v>131</v>
+      </c>
+      <c r="D51" s="6"/>
+      <c r="E51" s="7"/>
+    </row>
+    <row r="52" ht="20.05" customHeight="1">
+      <c r="A52" t="s" s="9">
+        <v>132</v>
+      </c>
+      <c r="B52" t="s" s="9">
+        <v>133</v>
+      </c>
+      <c r="C52" t="s" s="9">
+        <v>134</v>
+      </c>
+      <c r="D52" s="6"/>
+      <c r="E52" s="7"/>
+    </row>
+    <row r="53" ht="20.05" customHeight="1">
+      <c r="A53" t="s" s="9">
+        <v>135</v>
+      </c>
+      <c r="B53" t="s" s="9">
+        <v>136</v>
+      </c>
+      <c r="C53" t="s" s="9">
+        <v>137</v>
+      </c>
+      <c r="D53" s="6"/>
+      <c r="E53" s="7"/>
+    </row>
+    <row r="54" ht="32.05" customHeight="1">
+      <c r="A54" t="s" s="9">
+        <v>138</v>
+      </c>
+      <c r="B54" t="s" s="9">
+        <v>139</v>
+      </c>
+      <c r="C54" t="s" s="9">
+        <v>140</v>
+      </c>
+      <c r="D54" s="6"/>
+      <c r="E54" s="7"/>
+    </row>
+    <row r="55" ht="20.05" customHeight="1">
+      <c r="A55" t="s" s="9">
+        <v>141</v>
+      </c>
+      <c r="B55" t="s" s="9">
+        <v>142</v>
+      </c>
+      <c r="C55" t="s" s="9">
+        <v>143</v>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="7"/>
+    </row>
+    <row r="56" ht="20.05" customHeight="1">
+      <c r="A56" t="s" s="9">
+        <v>141</v>
+      </c>
+      <c r="B56" t="s" s="9">
+        <v>144</v>
+      </c>
+      <c r="C56" t="s" s="9">
+        <v>145</v>
+      </c>
+      <c r="D56" s="6"/>
+      <c r="E56" s="7"/>
+    </row>
+    <row r="57" ht="20.05" customHeight="1">
+      <c r="A57" t="s" s="9">
+        <v>141</v>
+      </c>
+      <c r="B57" t="s" s="9">
+        <v>146</v>
+      </c>
+      <c r="C57" t="s" s="9">
+        <v>147</v>
+      </c>
+      <c r="D57" s="6"/>
+      <c r="E57" s="7"/>
+    </row>
+    <row r="58" ht="20.05" customHeight="1">
+      <c r="A58" t="s" s="9">
+        <v>141</v>
+      </c>
+      <c r="B58" t="s" s="9">
+        <v>148</v>
+      </c>
+      <c r="C58" t="s" s="9">
+        <v>149</v>
+      </c>
+      <c r="D58" s="6"/>
+      <c r="E58" s="7"/>
+    </row>
+    <row r="59" ht="32.05" customHeight="1">
+      <c r="A59" t="s" s="9">
+        <v>150</v>
+      </c>
+      <c r="B59" t="s" s="9">
+        <v>151</v>
+      </c>
+      <c r="C59" t="s" s="9">
+        <v>152</v>
+      </c>
+      <c r="D59" s="6"/>
+      <c r="E59" s="7"/>
+    </row>
+    <row r="60" ht="32.05" customHeight="1">
+      <c r="A60" t="s" s="9">
+        <v>153</v>
+      </c>
+      <c r="B60" t="s" s="9">
+        <v>154</v>
+      </c>
+      <c r="C60" t="s" s="9">
+        <v>155</v>
+      </c>
+      <c r="D60" s="6"/>
+      <c r="E60" s="7"/>
+    </row>
+    <row r="61" ht="20.05" customHeight="1">
+      <c r="A61" t="s" s="9">
+        <v>156</v>
+      </c>
+      <c r="B61" t="s" s="9">
+        <v>157</v>
+      </c>
+      <c r="C61" t="s" s="9">
+        <v>158</v>
+      </c>
+      <c r="D61" s="6"/>
+      <c r="E61" s="7"/>
+    </row>
+    <row r="62" ht="20.05" customHeight="1">
+      <c r="A62" t="s" s="9">
+        <v>159</v>
+      </c>
+      <c r="B62" t="s" s="9">
+        <v>160</v>
+      </c>
+      <c r="C62" t="s" s="9">
+        <v>161</v>
+      </c>
+      <c r="D62" s="10"/>
+      <c r="E62" s="11"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27331a7db5370134479f43b43e8"/>
-    <hyperlink ref="C3" r:id="rId2" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e8dd4db47e7177c63b0b7d53"/>
+    <hyperlink ref="C2" r:id="rId1" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e8dd4db47e7177c63b0b7d53"/>
+    <hyperlink ref="C3" r:id="rId2" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27331a7db5370134479f43b43e8"/>
     <hyperlink ref="C4" r:id="rId3" location="" tooltip="" display="https://www.rockaxis.com/img/newsList/2907951.jpg"/>
-    <hyperlink ref="C5" r:id="rId4" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dbeec63ad914c973e75c24df"/>
-    <hyperlink ref="C6" r:id="rId5" location="" tooltip="" display="https://vinilosargentinos.com/wp-content/uploads/2025/01/y-1.jpg"/>
-    <hyperlink ref="C7" r:id="rId6" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273557e06d39588819e7a322817"/>
-    <hyperlink ref="C8" r:id="rId7" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273eb7f16ce83db71362ecb0cb5"/>
-    <hyperlink ref="C9" r:id="rId8" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27314653b83cd7d851accdb5142"/>
-    <hyperlink ref="C10" r:id="rId9" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739164bafe9aaa168d93f4816a"/>
-    <hyperlink ref="C11" r:id="rId10" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273b760d33bf5c940e64dccf56e"/>
-    <hyperlink ref="C12" r:id="rId11" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e9ce6d751caa0aa5596af3ca"/>
-    <hyperlink ref="C13" r:id="rId12" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273cee68f3a6e7d93b888461ae0"/>
-    <hyperlink ref="C14" r:id="rId13" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732ef0bb0bcabb4449cc0b2d0d"/>
-    <hyperlink ref="C15" r:id="rId14" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732172b607853fa89cefa2beb4"/>
-    <hyperlink ref="C16" r:id="rId15" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732f8790ed72296c2614607575"/>
-    <hyperlink ref="C17" r:id="rId16" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733e030a7e606959674643d274"/>
-    <hyperlink ref="C18" r:id="rId17" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80"/>
-    <hyperlink ref="C19" r:id="rId18" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b"/>
-    <hyperlink ref="C20" r:id="rId19" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279"/>
-    <hyperlink ref="C21" r:id="rId20" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7"/>
-    <hyperlink ref="C22" r:id="rId21" location="" tooltip="" display="https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg"/>
-    <hyperlink ref="C23" r:id="rId22" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473"/>
-    <hyperlink ref="C24" r:id="rId23" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4"/>
-    <hyperlink ref="C25" r:id="rId24" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f"/>
-    <hyperlink ref="C26" r:id="rId25" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff"/>
-    <hyperlink ref="C27" r:id="rId26" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca"/>
-    <hyperlink ref="C28" r:id="rId27" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e"/>
-    <hyperlink ref="C29" r:id="rId28" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400"/>
-    <hyperlink ref="C30" r:id="rId29" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08"/>
-    <hyperlink ref="C31" r:id="rId30" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3"/>
-    <hyperlink ref="C32" r:id="rId31" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135"/>
-    <hyperlink ref="C33" r:id="rId32" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87"/>
-    <hyperlink ref="C34" r:id="rId33" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419"/>
-    <hyperlink ref="C35" r:id="rId34" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537"/>
-    <hyperlink ref="C36" r:id="rId35" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02"/>
-    <hyperlink ref="C37" r:id="rId36" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733935c39bea149ac15c83c41a"/>
-    <hyperlink ref="C38" r:id="rId37" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730320739a960dd4821b2aeaf1"/>
-    <hyperlink ref="C39" r:id="rId38" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273139d10e0ae979a7b4a811140"/>
-    <hyperlink ref="C40" r:id="rId39" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733443d9c76e9713a5986c983c"/>
-    <hyperlink ref="C41" r:id="rId40" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dfc72dec3da479c81c575551"/>
-    <hyperlink ref="C42" r:id="rId41" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c3780b28120b1bc2869a2ca7"/>
-    <hyperlink ref="C43" r:id="rId42" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737e553e1367924fa3429a692c"/>
-    <hyperlink ref="C44" r:id="rId43" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e28947f6ad2f100af9c1965a"/>
-    <hyperlink ref="C45" r:id="rId44" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273d8abc667a17dab2e1a6bd44e"/>
-    <hyperlink ref="C46" r:id="rId45" location="" tooltip="" display="https://i.discogs.com/JGlQq8Q4mFy5ZdAmZrm52sAPV7S3gqKvmhCAfkyeJac/rs:fit/g:sm/q:40/h:300/w:300/czM6Ly9kaXNjb2dz/LWRhdGFiYXNlLWlt/YWdlcy9SLTk3ODI5/MzItMTYwNTU4NDg4/OC0zNDk2LmpwZWc.jpeg"/>
-    <hyperlink ref="C47" r:id="rId46" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273804c1bb88d714079e12d80e1"/>
-    <hyperlink ref="C48" r:id="rId47" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730cef6c8d0af7bde036793c4a"/>
-    <hyperlink ref="C49" r:id="rId48" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739934f74a9f25f2d4d0d9509e"/>
+    <hyperlink ref="C5" r:id="rId4" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2734ae1c4c5c45aabe565499163"/>
+    <hyperlink ref="C6" r:id="rId5" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2738895ff0f90525f4aa9437c27"/>
+    <hyperlink ref="C7" r:id="rId6" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dbeec63ad914c973e75c24df"/>
+    <hyperlink ref="C8" r:id="rId7" location="" tooltip="" display="https://vinilosargentinos.com/wp-content/uploads/2025/01/y-1.jpg"/>
+    <hyperlink ref="C9" r:id="rId8" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273557e06d39588819e7a322817"/>
+    <hyperlink ref="C10" r:id="rId9" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273eb7f16ce83db71362ecb0cb5"/>
+    <hyperlink ref="C11" r:id="rId10" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27314653b83cd7d851accdb5142"/>
+    <hyperlink ref="C12" r:id="rId11" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885"/>
+    <hyperlink ref="C13" r:id="rId12" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab"/>
+    <hyperlink ref="C14" r:id="rId13" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27392441ecd34874c2bc4f19144"/>
+    <hyperlink ref="C15" r:id="rId14" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739164bafe9aaa168d93f4816a"/>
+    <hyperlink ref="C16" r:id="rId15" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e21cc1db05580b6f2d2a3b6e"/>
+    <hyperlink ref="C17" r:id="rId16" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273b760d33bf5c940e64dccf56e"/>
+    <hyperlink ref="C18" r:id="rId17" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e9ce6d751caa0aa5596af3ca"/>
+    <hyperlink ref="C19" r:id="rId18" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739b9b36b0e22870b9f542d937"/>
+    <hyperlink ref="C20" r:id="rId19" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7"/>
+    <hyperlink ref="C21" r:id="rId20" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273cee68f3a6e7d93b888461ae0"/>
+    <hyperlink ref="C22" r:id="rId21" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732ef0bb0bcabb4449cc0b2d0d"/>
+    <hyperlink ref="C23" r:id="rId22" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732172b607853fa89cefa2beb4"/>
+    <hyperlink ref="C24" r:id="rId23" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2732f8790ed72296c2614607575"/>
+    <hyperlink ref="C25" r:id="rId24" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80"/>
+    <hyperlink ref="C26" r:id="rId25" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733e030a7e606959674643d274"/>
+    <hyperlink ref="C27" r:id="rId26" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b"/>
+    <hyperlink ref="C28" r:id="rId27" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279"/>
+    <hyperlink ref="C29" r:id="rId28" location="" tooltip="" display="https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg"/>
+    <hyperlink ref="C30" r:id="rId29" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473"/>
+    <hyperlink ref="C31" r:id="rId30" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4"/>
+    <hyperlink ref="C32" r:id="rId31" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f"/>
+    <hyperlink ref="C33" r:id="rId32" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff"/>
+    <hyperlink ref="C34" r:id="rId33" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca"/>
+    <hyperlink ref="C35" r:id="rId34" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e"/>
+    <hyperlink ref="C36" r:id="rId35" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400"/>
+    <hyperlink ref="C37" r:id="rId36" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08"/>
+    <hyperlink ref="C38" r:id="rId37" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3"/>
+    <hyperlink ref="C39" r:id="rId38" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135"/>
+    <hyperlink ref="C40" r:id="rId39" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27350db5a166ea23d5d6c4cd387"/>
+    <hyperlink ref="C41" r:id="rId40" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273ef221258ca5f3e223937d408"/>
+    <hyperlink ref="C42" r:id="rId41" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87"/>
+    <hyperlink ref="C43" r:id="rId42" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419"/>
+    <hyperlink ref="C44" r:id="rId43" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537"/>
+    <hyperlink ref="C45" r:id="rId44" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02"/>
+    <hyperlink ref="C46" r:id="rId45" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492"/>
+    <hyperlink ref="C47" r:id="rId46" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273b57713d0fe3553a087419f8f"/>
+    <hyperlink ref="C48" r:id="rId47" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273056e90910cbaf5c5b892aeba"/>
+    <hyperlink ref="C49" r:id="rId48" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733935c39bea149ac15c83c41a"/>
+    <hyperlink ref="C50" r:id="rId49" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730320739a960dd4821b2aeaf1"/>
+    <hyperlink ref="C51" r:id="rId50" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273139d10e0ae979a7b4a811140"/>
+    <hyperlink ref="C52" r:id="rId51" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733443d9c76e9713a5986c983c"/>
+    <hyperlink ref="C53" r:id="rId52" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273ac84ce59dc5d49c81dc9d8fb"/>
+    <hyperlink ref="C54" r:id="rId53" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dfc72dec3da479c81c575551"/>
+    <hyperlink ref="C55" r:id="rId54" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273c3780b28120b1bc2869a2ca7"/>
+    <hyperlink ref="C56" r:id="rId55" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737e553e1367924fa3429a692c"/>
+    <hyperlink ref="C57" r:id="rId56" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e28947f6ad2f100af9c1965a"/>
+    <hyperlink ref="C58" r:id="rId57" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273d8abc667a17dab2e1a6bd44e"/>
+    <hyperlink ref="C59" r:id="rId58" location="" tooltip="" display="https://i.discogs.com/JGlQq8Q4mFy5ZdAmZrm52sAPV7S3gqKvmhCAfkyeJac/rs:fit/g:sm/q:40/h:300/w:300/czM6Ly9kaXNjb2dz/LWRhdGFiYXNlLWlt/YWdlcy9SLTk3ODI5/MzItMTYwNTU4NDg4/OC0zNDk2LmpwZWc.jpeg"/>
+    <hyperlink ref="C60" r:id="rId59" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273804c1bb88d714079e12d80e1"/>
+    <hyperlink ref="C61" r:id="rId60" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2730cef6c8d0af7bde036793c4a"/>
+    <hyperlink ref="C62" r:id="rId61" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739934f74a9f25f2d4d0d9509e"/>
   </hyperlinks>
   <pageMargins left="0.5" right="0.5" top="0.75" bottom="0.75" header="0.277778" footer="0.277778"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="72" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
Corrijo orden por nombre de disco
</commit_message>
<xml_diff>
--- a/public/discos.xlsx
+++ b/public/discos.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="161">
   <si>
     <t>Artista</t>
   </si>
@@ -149,7 +149,35 @@
     </r>
   </si>
   <si>
-    <t>Cerati - Melero</t>
+    <t>Cerati Gustavo</t>
+  </si>
+  <si>
+    <t>Amor Amarillo</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885</t>
+    </r>
+  </si>
+  <si>
+    <t>Bocanada</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="14"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab</t>
+    </r>
   </si>
   <si>
     <t>Colores Santos</t>
@@ -166,9 +194,6 @@
     </r>
   </si>
   <si>
-    <t>Cerati Gustavo</t>
-  </si>
-  <si>
     <t>Fuerza Natural</t>
   </si>
   <si>
@@ -183,7 +208,7 @@
     </r>
   </si>
   <si>
-    <t>Amor Amarillo</t>
+    <t>Siempre es Hoy</t>
   </si>
   <si>
     <r>
@@ -193,11 +218,28 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885</t>
-    </r>
-  </si>
-  <si>
-    <t>Bocanada</t>
+      <t>https://i.scdn.co/image/ab67616d0000b27392441ecd34874c2bc4f19144</t>
+    </r>
+  </si>
+  <si>
+    <t>Coldplay</t>
+  </si>
+  <si>
+    <t>Parachutes</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2739164bafe9aaa168d93f4816a</t>
+    </r>
+  </si>
+  <si>
+    <t>Viva la Vida</t>
   </si>
   <si>
     <r>
@@ -207,11 +249,45 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab</t>
-    </r>
-  </si>
-  <si>
-    <t>Siempre es Hoy</t>
+      <t>https://i.scdn.co/image/ab67616d0000b273e21cc1db05580b6f2d2a3b6e</t>
+    </r>
+  </si>
+  <si>
+    <t>Conociendo Rusia</t>
+  </si>
+  <si>
+    <t>Cabildo y Juramento</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273b760d33bf5c940e64dccf56e</t>
+    </r>
+  </si>
+  <si>
+    <t>Jet Love</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e9ce6d751caa0aa5596af3ca</t>
+    </r>
+  </si>
+  <si>
+    <t>Daft Punk</t>
+  </si>
+  <si>
+    <t>Random Access Memory</t>
   </si>
   <si>
     <r>
@@ -221,28 +297,342 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b27392441ecd34874c2bc4f19144</t>
-    </r>
-  </si>
-  <si>
-    <t>Coldplay</t>
-  </si>
-  <si>
-    <t>Parachutes</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2739164bafe9aaa168d93f4816a</t>
-    </r>
-  </si>
-  <si>
-    <t>Viva la Vida</t>
+      <t>https://i.scdn.co/image/ab67616d0000b2739b9b36b0e22870b9f542d937</t>
+    </r>
+  </si>
+  <si>
+    <t>David Guetta</t>
+  </si>
+  <si>
+    <t>Nothing but the beat</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7</t>
+    </r>
+  </si>
+  <si>
+    <t>Deep Purple</t>
+  </si>
+  <si>
+    <t>In Rock</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273cee68f3a6e7d93b888461ae0</t>
+    </r>
+  </si>
+  <si>
+    <t>Denis Sergio</t>
+  </si>
+  <si>
+    <t>Sergio Denis</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2732ef0bb0bcabb4449cc0b2d0d</t>
+    </r>
+  </si>
+  <si>
+    <t>Dua Lipa</t>
+  </si>
+  <si>
+    <t>Future Nostalgia</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2732172b607853fa89cefa2beb4</t>
+    </r>
+  </si>
+  <si>
+    <t>Radical Optimism</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2732f8790ed72296c2614607575</t>
+    </r>
+  </si>
+  <si>
+    <t>Fito Paez</t>
+  </si>
+  <si>
+    <t>Giros</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80</t>
+    </r>
+  </si>
+  <si>
+    <t>Foreigner</t>
+  </si>
+  <si>
+    <t>Agent Provocateur</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2733e030a7e606959674643d274</t>
+    </r>
+  </si>
+  <si>
+    <t>Gorillaz</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b</t>
+    </r>
+  </si>
+  <si>
+    <t>Green day</t>
+  </si>
+  <si>
+    <t>American Idiot</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279</t>
+    </r>
+  </si>
+  <si>
+    <t>Harrison George</t>
+  </si>
+  <si>
+    <t>Lo mejor de George Harrison</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg</t>
+    </r>
+  </si>
+  <si>
+    <t>Kool &amp; the Gang</t>
+  </si>
+  <si>
+    <t>Celebrate!</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473</t>
+    </r>
+  </si>
+  <si>
+    <t>Lali</t>
+  </si>
+  <si>
+    <t>No vayas a atender cuando el demonio llama</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4</t>
+    </r>
+  </si>
+  <si>
+    <t>Led Zeppelin</t>
+  </si>
+  <si>
+    <t>Led Zeppelin I</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f</t>
+    </r>
+  </si>
+  <si>
+    <t>Miguel Luis</t>
+  </si>
+  <si>
+    <t>Aries</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff</t>
+    </r>
+  </si>
+  <si>
+    <t>Busca una mujer</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca</t>
+    </r>
+  </si>
+  <si>
+    <t>Miranda!</t>
+  </si>
+  <si>
+    <t>Nuevo Hotel Miranda!</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e</t>
+    </r>
+  </si>
+  <si>
+    <t>Muse</t>
+  </si>
+  <si>
+    <t>Black Holes and Revelation</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400</t>
+    </r>
+  </si>
+  <si>
+    <t>No te Va Gustar</t>
+  </si>
+  <si>
+    <t>El calor del pleno invierno</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08</t>
+    </r>
+  </si>
+  <si>
+    <t>Por lo menos hoy</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3</t>
+    </r>
+  </si>
+  <si>
+    <t>Palito Ortega</t>
+  </si>
+  <si>
+    <t>Palito Ortega Nº 21</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135</t>
+    </r>
+  </si>
+  <si>
+    <t>Pescado Rabioso</t>
+  </si>
+  <si>
+    <t>Artaud</t>
   </si>
   <si>
     <r>
@@ -252,45 +642,14 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273e21cc1db05580b6f2d2a3b6e</t>
-    </r>
-  </si>
-  <si>
-    <t>Conociendo Rusia</t>
-  </si>
-  <si>
-    <t>Cabildo y Juramento</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273b760d33bf5c940e64dccf56e</t>
-    </r>
-  </si>
-  <si>
-    <t>Jet Love</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273e9ce6d751caa0aa5596af3ca</t>
-    </r>
-  </si>
-  <si>
-    <t>Daft Punk</t>
-  </si>
-  <si>
-    <t>Random Access Memory</t>
+      <t>https://i.scdn.co/image/ab67616d0000b27350db5a166ea23d5d6c4cd387</t>
+    </r>
+  </si>
+  <si>
+    <t>Pointed Sisters</t>
+  </si>
+  <si>
+    <t>Contact</t>
   </si>
   <si>
     <r>
@@ -300,342 +659,14 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2739b9b36b0e22870b9f542d937</t>
-    </r>
-  </si>
-  <si>
-    <t>David Guetta</t>
-  </si>
-  <si>
-    <t>Nothing but the beat</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b27354e095b51d4ba95496cd60d7</t>
-    </r>
-  </si>
-  <si>
-    <t>Deep Purple</t>
-  </si>
-  <si>
-    <t>In Rock</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273cee68f3a6e7d93b888461ae0</t>
-    </r>
-  </si>
-  <si>
-    <t>Denis Sergio</t>
-  </si>
-  <si>
-    <t>Sergio Denis</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2732ef0bb0bcabb4449cc0b2d0d</t>
-    </r>
-  </si>
-  <si>
-    <t>Dua Lipa</t>
-  </si>
-  <si>
-    <t>Future Nostalgia</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2732172b607853fa89cefa2beb4</t>
-    </r>
-  </si>
-  <si>
-    <t>Radical Optimism</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2732f8790ed72296c2614607575</t>
-    </r>
-  </si>
-  <si>
-    <t>Fito Paez</t>
-  </si>
-  <si>
-    <t>Giros</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273921417baf700cc9da1d43b80</t>
-    </r>
-  </si>
-  <si>
-    <t>Foreigner</t>
-  </si>
-  <si>
-    <t>Agent Provocateur</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2733e030a7e606959674643d274</t>
-    </r>
-  </si>
-  <si>
-    <t>Gorillaz</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273c73a7bb15f43bae86215934b</t>
-    </r>
-  </si>
-  <si>
-    <t>Green day</t>
-  </si>
-  <si>
-    <t>American Idiot</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2730b07888116d8bb9161228279</t>
-    </r>
-  </si>
-  <si>
-    <t>Harrison George</t>
-  </si>
-  <si>
-    <t>Lo mejor de George Harrison</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://m.media-amazon.com/images/I/71iibB76ztL._UF1000,1000_QL80_.jpg</t>
-    </r>
-  </si>
-  <si>
-    <t>Kool &amp; the Gang</t>
-  </si>
-  <si>
-    <t>Celebrate!</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273887b7c596249f628db6c6473</t>
-    </r>
-  </si>
-  <si>
-    <t>Lali</t>
-  </si>
-  <si>
-    <t>No vayas a atender cuando el demonio llama</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273f6ed36ac805c4d231e0537f4</t>
-    </r>
-  </si>
-  <si>
-    <t>Led Zeppelin</t>
-  </si>
-  <si>
-    <t>Led Zeppelin I</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273c77c73285cc5cb64d97e1b0f</t>
-    </r>
-  </si>
-  <si>
-    <t>Miguel Luis</t>
-  </si>
-  <si>
-    <t>Aries</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273780268564c65ca302786e6ff</t>
-    </r>
-  </si>
-  <si>
-    <t>Busca una mujer</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2737144526743136029a4d61aca</t>
-    </r>
-  </si>
-  <si>
-    <t>Miranda!</t>
-  </si>
-  <si>
-    <t>Nuevo Hotel Miranda!</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273932207d3eed1cae5f0b81a0e</t>
-    </r>
-  </si>
-  <si>
-    <t>Muse</t>
-  </si>
-  <si>
-    <t>Black Holes and Revelation</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b27328933b808bfb4cbbd0385400</t>
-    </r>
-  </si>
-  <si>
-    <t>No te Va Gustar</t>
-  </si>
-  <si>
-    <t>El calor del pleno invierno</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273e73cfb1faa1d5bde8cc96c08</t>
-    </r>
-  </si>
-  <si>
-    <t>Por lo menos hoy</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273fa9302d9b82dce4d3ed429e3</t>
-    </r>
-  </si>
-  <si>
-    <t>Palito Ortega</t>
-  </si>
-  <si>
-    <t>Palito Ortega Nº 21</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135</t>
-    </r>
-  </si>
-  <si>
-    <t>Pescado Rabioso</t>
-  </si>
-  <si>
-    <t>Artaud</t>
+      <t>https://i.scdn.co/image/ab67616d0000b273ef221258ca5f3e223937d408</t>
+    </r>
+  </si>
+  <si>
+    <t>Queen</t>
+  </si>
+  <si>
+    <t>A day at the Races</t>
   </si>
   <si>
     <r>
@@ -645,28 +676,50 @@
         <color indexed="14"/>
         <rFont val="Helvetica Neue"/>
       </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b27350db5a166ea23d5d6c4cd387</t>
-    </r>
-  </si>
-  <si>
-    <t>Pointed Sisters</t>
-  </si>
-  <si>
-    <t>Contact</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="14"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273ef221258ca5f3e223937d408</t>
-    </r>
-  </si>
-  <si>
-    <t>Queen</t>
+      <t>https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492</t>
+    </r>
+  </si>
+  <si>
+    <t>A Kind of Magic</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419</t>
+    </r>
+  </si>
+  <si>
+    <t>A Night at the Opera</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537</t>
+    </r>
+  </si>
+  <si>
+    <t>Flashgordon</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <u val="single"/>
+        <sz val="10"/>
+        <color indexed="8"/>
+        <rFont val="Helvetica Neue"/>
+      </rPr>
+      <t>https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02</t>
+    </r>
   </si>
   <si>
     <r>
@@ -677,62 +730,6 @@
         <rFont val="Helvetica Neue"/>
       </rPr>
       <t>https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87</t>
-    </r>
-  </si>
-  <si>
-    <t>A Kind of Magic</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419</t>
-    </r>
-  </si>
-  <si>
-    <t>A Night at the Opera</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537</t>
-    </r>
-  </si>
-  <si>
-    <t>Flashgordon</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="8"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02</t>
-    </r>
-  </si>
-  <si>
-    <t>A day at the Races</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <u val="single"/>
-        <sz val="10"/>
-        <color indexed="14"/>
-        <rFont val="Helvetica Neue"/>
-      </rPr>
-      <t>https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492</t>
     </r>
   </si>
   <si>
@@ -2403,410 +2400,410 @@
     </row>
     <row r="11" ht="20.05" customHeight="1">
       <c r="A11" t="s" s="9">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s" s="9">
         <v>27</v>
       </c>
-      <c r="B11" t="s" s="9">
+      <c r="C11" t="s" s="9">
         <v>28</v>
-      </c>
-      <c r="C11" t="s" s="9">
-        <v>29</v>
       </c>
       <c r="D11" s="6"/>
       <c r="E11" s="7"/>
     </row>
     <row r="12" ht="20.05" customHeight="1">
       <c r="A12" t="s" s="9">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s" s="9">
+        <v>29</v>
+      </c>
+      <c r="C12" t="s" s="9">
         <v>30</v>
-      </c>
-      <c r="C12" t="s" s="9">
-        <v>31</v>
       </c>
       <c r="D12" s="6"/>
       <c r="E12" s="7"/>
     </row>
     <row r="13" ht="20.05" customHeight="1">
       <c r="A13" t="s" s="9">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s" s="9">
+        <v>31</v>
+      </c>
+      <c r="C13" t="s" s="9">
         <v>32</v>
-      </c>
-      <c r="C13" t="s" s="9">
-        <v>33</v>
       </c>
       <c r="D13" s="6"/>
       <c r="E13" s="7"/>
     </row>
     <row r="14" ht="20.05" customHeight="1">
       <c r="A14" t="s" s="9">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s" s="9">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s" s="9">
         <v>34</v>
-      </c>
-      <c r="C14" t="s" s="9">
-        <v>35</v>
       </c>
       <c r="D14" s="6"/>
       <c r="E14" s="7"/>
     </row>
     <row r="15" ht="20.05" customHeight="1">
       <c r="A15" t="s" s="9">
+        <v>35</v>
+      </c>
+      <c r="B15" t="s" s="9">
         <v>36</v>
       </c>
-      <c r="B15" t="s" s="9">
+      <c r="C15" t="s" s="9">
         <v>37</v>
-      </c>
-      <c r="C15" t="s" s="9">
-        <v>38</v>
       </c>
       <c r="D15" s="6"/>
       <c r="E15" s="7"/>
     </row>
     <row r="16" ht="20.05" customHeight="1">
       <c r="A16" t="s" s="9">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s" s="9">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s" s="9">
         <v>39</v>
-      </c>
-      <c r="C16" t="s" s="9">
-        <v>40</v>
       </c>
       <c r="D16" s="6"/>
       <c r="E16" s="7"/>
     </row>
     <row r="17" ht="32.05" customHeight="1">
       <c r="A17" t="s" s="9">
+        <v>40</v>
+      </c>
+      <c r="B17" t="s" s="9">
         <v>41</v>
       </c>
-      <c r="B17" t="s" s="9">
+      <c r="C17" t="s" s="9">
         <v>42</v>
-      </c>
-      <c r="C17" t="s" s="9">
-        <v>43</v>
       </c>
       <c r="D17" s="6"/>
       <c r="E17" s="7"/>
     </row>
     <row r="18" ht="20.05" customHeight="1">
       <c r="A18" t="s" s="9">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s" s="9">
+        <v>43</v>
+      </c>
+      <c r="C18" t="s" s="9">
         <v>44</v>
-      </c>
-      <c r="C18" t="s" s="9">
-        <v>45</v>
       </c>
       <c r="D18" s="6"/>
       <c r="E18" s="7"/>
     </row>
     <row r="19" ht="20.05" customHeight="1">
       <c r="A19" t="s" s="9">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s" s="9">
         <v>46</v>
       </c>
-      <c r="B19" t="s" s="9">
+      <c r="C19" t="s" s="9">
         <v>47</v>
-      </c>
-      <c r="C19" t="s" s="9">
-        <v>48</v>
       </c>
       <c r="D19" s="6"/>
       <c r="E19" s="7"/>
     </row>
     <row r="20" ht="32.05" customHeight="1">
       <c r="A20" t="s" s="9">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s" s="9">
         <v>49</v>
       </c>
-      <c r="B20" t="s" s="9">
+      <c r="C20" t="s" s="9">
         <v>50</v>
-      </c>
-      <c r="C20" t="s" s="9">
-        <v>51</v>
       </c>
       <c r="D20" s="6"/>
       <c r="E20" s="7"/>
     </row>
     <row r="21" ht="20.05" customHeight="1">
       <c r="A21" t="s" s="9">
+        <v>51</v>
+      </c>
+      <c r="B21" t="s" s="9">
         <v>52</v>
       </c>
-      <c r="B21" t="s" s="9">
+      <c r="C21" t="s" s="9">
         <v>53</v>
-      </c>
-      <c r="C21" t="s" s="9">
-        <v>54</v>
       </c>
       <c r="D21" s="6"/>
       <c r="E21" s="7"/>
     </row>
     <row r="22" ht="20.05" customHeight="1">
       <c r="A22" t="s" s="9">
+        <v>54</v>
+      </c>
+      <c r="B22" t="s" s="9">
         <v>55</v>
       </c>
-      <c r="B22" t="s" s="9">
+      <c r="C22" t="s" s="9">
         <v>56</v>
-      </c>
-      <c r="C22" t="s" s="9">
-        <v>57</v>
       </c>
       <c r="D22" s="6"/>
       <c r="E22" s="7"/>
     </row>
     <row r="23" ht="20.05" customHeight="1">
       <c r="A23" t="s" s="9">
+        <v>57</v>
+      </c>
+      <c r="B23" t="s" s="9">
         <v>58</v>
       </c>
-      <c r="B23" t="s" s="9">
+      <c r="C23" t="s" s="9">
         <v>59</v>
-      </c>
-      <c r="C23" t="s" s="9">
-        <v>60</v>
       </c>
       <c r="D23" s="6"/>
       <c r="E23" s="7"/>
     </row>
     <row r="24" ht="20.05" customHeight="1">
       <c r="A24" t="s" s="9">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B24" t="s" s="9">
+        <v>60</v>
+      </c>
+      <c r="C24" t="s" s="9">
         <v>61</v>
-      </c>
-      <c r="C24" t="s" s="9">
-        <v>62</v>
       </c>
       <c r="D24" s="6"/>
       <c r="E24" s="7"/>
     </row>
     <row r="25" ht="20.05" customHeight="1">
       <c r="A25" t="s" s="9">
+        <v>62</v>
+      </c>
+      <c r="B25" t="s" s="9">
         <v>63</v>
       </c>
-      <c r="B25" t="s" s="9">
+      <c r="C25" t="s" s="9">
         <v>64</v>
-      </c>
-      <c r="C25" t="s" s="9">
-        <v>65</v>
       </c>
       <c r="D25" s="6"/>
       <c r="E25" s="7"/>
     </row>
     <row r="26" ht="20.05" customHeight="1">
       <c r="A26" t="s" s="9">
+        <v>65</v>
+      </c>
+      <c r="B26" t="s" s="9">
         <v>66</v>
       </c>
-      <c r="B26" t="s" s="9">
+      <c r="C26" t="s" s="9">
         <v>67</v>
-      </c>
-      <c r="C26" t="s" s="9">
-        <v>68</v>
       </c>
       <c r="D26" s="6"/>
       <c r="E26" s="7"/>
     </row>
     <row r="27" ht="20.05" customHeight="1">
       <c r="A27" t="s" s="9">
+        <v>68</v>
+      </c>
+      <c r="B27" t="s" s="9">
+        <v>68</v>
+      </c>
+      <c r="C27" t="s" s="9">
         <v>69</v>
-      </c>
-      <c r="B27" t="s" s="9">
-        <v>69</v>
-      </c>
-      <c r="C27" t="s" s="9">
-        <v>70</v>
       </c>
       <c r="D27" s="6"/>
       <c r="E27" s="7"/>
     </row>
     <row r="28" ht="20.05" customHeight="1">
       <c r="A28" t="s" s="9">
+        <v>70</v>
+      </c>
+      <c r="B28" t="s" s="9">
         <v>71</v>
       </c>
-      <c r="B28" t="s" s="9">
+      <c r="C28" t="s" s="9">
         <v>72</v>
-      </c>
-      <c r="C28" t="s" s="9">
-        <v>73</v>
       </c>
       <c r="D28" s="6"/>
       <c r="E28" s="7"/>
     </row>
     <row r="29" ht="32.05" customHeight="1">
       <c r="A29" t="s" s="9">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s" s="9">
         <v>74</v>
       </c>
-      <c r="B29" t="s" s="9">
+      <c r="C29" t="s" s="9">
         <v>75</v>
-      </c>
-      <c r="C29" t="s" s="9">
-        <v>76</v>
       </c>
       <c r="D29" s="6"/>
       <c r="E29" s="7"/>
     </row>
     <row r="30" ht="20.05" customHeight="1">
       <c r="A30" t="s" s="9">
+        <v>76</v>
+      </c>
+      <c r="B30" t="s" s="9">
         <v>77</v>
       </c>
-      <c r="B30" t="s" s="9">
+      <c r="C30" t="s" s="9">
         <v>78</v>
-      </c>
-      <c r="C30" t="s" s="9">
-        <v>79</v>
       </c>
       <c r="D30" s="6"/>
       <c r="E30" s="7"/>
     </row>
     <row r="31" ht="44.05" customHeight="1">
       <c r="A31" t="s" s="9">
+        <v>79</v>
+      </c>
+      <c r="B31" t="s" s="9">
         <v>80</v>
       </c>
-      <c r="B31" t="s" s="9">
+      <c r="C31" t="s" s="9">
         <v>81</v>
-      </c>
-      <c r="C31" t="s" s="9">
-        <v>82</v>
       </c>
       <c r="D31" s="6"/>
       <c r="E31" s="7"/>
     </row>
     <row r="32" ht="20.05" customHeight="1">
       <c r="A32" t="s" s="9">
+        <v>82</v>
+      </c>
+      <c r="B32" t="s" s="9">
         <v>83</v>
       </c>
-      <c r="B32" t="s" s="9">
+      <c r="C32" t="s" s="9">
         <v>84</v>
-      </c>
-      <c r="C32" t="s" s="9">
-        <v>85</v>
       </c>
       <c r="D32" s="6"/>
       <c r="E32" s="7"/>
     </row>
     <row r="33" ht="20.05" customHeight="1">
       <c r="A33" t="s" s="9">
+        <v>85</v>
+      </c>
+      <c r="B33" t="s" s="9">
         <v>86</v>
       </c>
-      <c r="B33" t="s" s="9">
+      <c r="C33" t="s" s="9">
         <v>87</v>
-      </c>
-      <c r="C33" t="s" s="9">
-        <v>88</v>
       </c>
       <c r="D33" s="6"/>
       <c r="E33" s="7"/>
     </row>
     <row r="34" ht="20.05" customHeight="1">
       <c r="A34" t="s" s="9">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B34" t="s" s="9">
+        <v>88</v>
+      </c>
+      <c r="C34" t="s" s="9">
         <v>89</v>
-      </c>
-      <c r="C34" t="s" s="9">
-        <v>90</v>
       </c>
       <c r="D34" s="6"/>
       <c r="E34" s="7"/>
     </row>
     <row r="35" ht="32.05" customHeight="1">
       <c r="A35" t="s" s="9">
+        <v>90</v>
+      </c>
+      <c r="B35" t="s" s="9">
         <v>91</v>
       </c>
-      <c r="B35" t="s" s="9">
+      <c r="C35" t="s" s="9">
         <v>92</v>
-      </c>
-      <c r="C35" t="s" s="9">
-        <v>93</v>
       </c>
       <c r="D35" s="6"/>
       <c r="E35" s="7"/>
     </row>
     <row r="36" ht="32.05" customHeight="1">
       <c r="A36" t="s" s="9">
+        <v>93</v>
+      </c>
+      <c r="B36" t="s" s="9">
         <v>94</v>
       </c>
-      <c r="B36" t="s" s="9">
+      <c r="C36" t="s" s="9">
         <v>95</v>
-      </c>
-      <c r="C36" t="s" s="9">
-        <v>96</v>
       </c>
       <c r="D36" s="6"/>
       <c r="E36" s="7"/>
     </row>
     <row r="37" ht="32.05" customHeight="1">
       <c r="A37" t="s" s="9">
+        <v>96</v>
+      </c>
+      <c r="B37" t="s" s="9">
         <v>97</v>
       </c>
-      <c r="B37" t="s" s="9">
+      <c r="C37" t="s" s="9">
         <v>98</v>
-      </c>
-      <c r="C37" t="s" s="9">
-        <v>99</v>
       </c>
       <c r="D37" s="6"/>
       <c r="E37" s="7"/>
     </row>
     <row r="38" ht="20.05" customHeight="1">
       <c r="A38" t="s" s="9">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B38" t="s" s="9">
+        <v>99</v>
+      </c>
+      <c r="C38" t="s" s="9">
         <v>100</v>
-      </c>
-      <c r="C38" t="s" s="9">
-        <v>101</v>
       </c>
       <c r="D38" s="6"/>
       <c r="E38" s="7"/>
     </row>
     <row r="39" ht="20.05" customHeight="1">
       <c r="A39" t="s" s="9">
+        <v>101</v>
+      </c>
+      <c r="B39" t="s" s="9">
         <v>102</v>
       </c>
-      <c r="B39" t="s" s="9">
+      <c r="C39" t="s" s="9">
         <v>103</v>
-      </c>
-      <c r="C39" t="s" s="9">
-        <v>104</v>
       </c>
       <c r="D39" s="6"/>
       <c r="E39" s="7"/>
     </row>
     <row r="40" ht="20.05" customHeight="1">
       <c r="A40" t="s" s="9">
+        <v>104</v>
+      </c>
+      <c r="B40" t="s" s="9">
         <v>105</v>
       </c>
-      <c r="B40" t="s" s="9">
+      <c r="C40" t="s" s="9">
         <v>106</v>
-      </c>
-      <c r="C40" t="s" s="9">
-        <v>107</v>
       </c>
       <c r="D40" s="6"/>
       <c r="E40" s="7"/>
     </row>
     <row r="41" ht="20.05" customHeight="1">
       <c r="A41" t="s" s="9">
+        <v>107</v>
+      </c>
+      <c r="B41" t="s" s="9">
         <v>108</v>
       </c>
-      <c r="B41" t="s" s="9">
+      <c r="C41" t="s" s="9">
         <v>109</v>
-      </c>
-      <c r="C41" t="s" s="9">
-        <v>110</v>
       </c>
       <c r="D41" s="6"/>
       <c r="E41" s="7"/>
     </row>
     <row r="42" ht="20.05" customHeight="1">
       <c r="A42" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B42" t="s" s="9">
         <v>111</v>
@@ -2819,7 +2816,7 @@
     </row>
     <row r="43" ht="20.05" customHeight="1">
       <c r="A43" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B43" t="s" s="9">
         <v>113</v>
@@ -2832,7 +2829,7 @@
     </row>
     <row r="44" ht="32.05" customHeight="1">
       <c r="A44" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B44" t="s" s="9">
         <v>115</v>
@@ -2845,7 +2842,7 @@
     </row>
     <row r="45" ht="20.05" customHeight="1">
       <c r="A45" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B45" t="s" s="9">
         <v>117</v>
@@ -2858,221 +2855,221 @@
     </row>
     <row r="46" ht="20.05" customHeight="1">
       <c r="A46" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B46" t="s" s="9">
+        <v>110</v>
+      </c>
+      <c r="C46" t="s" s="9">
         <v>119</v>
-      </c>
-      <c r="C46" t="s" s="9">
-        <v>120</v>
       </c>
       <c r="D46" s="6"/>
       <c r="E46" s="7"/>
     </row>
     <row r="47" ht="20.05" customHeight="1">
       <c r="A47" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B47" t="s" s="9">
+        <v>120</v>
+      </c>
+      <c r="C47" t="s" s="9">
         <v>121</v>
-      </c>
-      <c r="C47" t="s" s="9">
-        <v>122</v>
       </c>
       <c r="D47" s="6"/>
       <c r="E47" s="7"/>
     </row>
     <row r="48" ht="20.05" customHeight="1">
       <c r="A48" t="s" s="9">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B48" t="s" s="9">
+        <v>122</v>
+      </c>
+      <c r="C48" t="s" s="9">
         <v>123</v>
-      </c>
-      <c r="C48" t="s" s="9">
-        <v>124</v>
       </c>
       <c r="D48" s="6"/>
       <c r="E48" s="7"/>
     </row>
     <row r="49" ht="20.05" customHeight="1">
       <c r="A49" t="s" s="9">
+        <v>124</v>
+      </c>
+      <c r="B49" t="s" s="9">
+        <v>124</v>
+      </c>
+      <c r="C49" t="s" s="9">
         <v>125</v>
-      </c>
-      <c r="B49" t="s" s="9">
-        <v>125</v>
-      </c>
-      <c r="C49" t="s" s="9">
-        <v>126</v>
       </c>
       <c r="D49" s="6"/>
       <c r="E49" s="7"/>
     </row>
     <row r="50" ht="20.05" customHeight="1">
       <c r="A50" t="s" s="9">
+        <v>126</v>
+      </c>
+      <c r="B50" t="s" s="9">
         <v>127</v>
       </c>
-      <c r="B50" t="s" s="9">
+      <c r="C50" t="s" s="9">
         <v>128</v>
-      </c>
-      <c r="C50" t="s" s="9">
-        <v>129</v>
       </c>
       <c r="D50" s="6"/>
       <c r="E50" s="7"/>
     </row>
     <row r="51" ht="20.05" customHeight="1">
       <c r="A51" t="s" s="9">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B51" t="s" s="9">
+        <v>129</v>
+      </c>
+      <c r="C51" t="s" s="9">
         <v>130</v>
-      </c>
-      <c r="C51" t="s" s="9">
-        <v>131</v>
       </c>
       <c r="D51" s="6"/>
       <c r="E51" s="7"/>
     </row>
     <row r="52" ht="20.05" customHeight="1">
       <c r="A52" t="s" s="9">
+        <v>131</v>
+      </c>
+      <c r="B52" t="s" s="9">
         <v>132</v>
       </c>
-      <c r="B52" t="s" s="9">
+      <c r="C52" t="s" s="9">
         <v>133</v>
-      </c>
-      <c r="C52" t="s" s="9">
-        <v>134</v>
       </c>
       <c r="D52" s="6"/>
       <c r="E52" s="7"/>
     </row>
     <row r="53" ht="20.05" customHeight="1">
       <c r="A53" t="s" s="9">
+        <v>134</v>
+      </c>
+      <c r="B53" t="s" s="9">
         <v>135</v>
       </c>
-      <c r="B53" t="s" s="9">
+      <c r="C53" t="s" s="9">
         <v>136</v>
-      </c>
-      <c r="C53" t="s" s="9">
-        <v>137</v>
       </c>
       <c r="D53" s="6"/>
       <c r="E53" s="7"/>
     </row>
     <row r="54" ht="32.05" customHeight="1">
       <c r="A54" t="s" s="9">
+        <v>137</v>
+      </c>
+      <c r="B54" t="s" s="9">
         <v>138</v>
       </c>
-      <c r="B54" t="s" s="9">
+      <c r="C54" t="s" s="9">
         <v>139</v>
-      </c>
-      <c r="C54" t="s" s="9">
-        <v>140</v>
       </c>
       <c r="D54" s="6"/>
       <c r="E54" s="7"/>
     </row>
     <row r="55" ht="20.05" customHeight="1">
       <c r="A55" t="s" s="9">
+        <v>140</v>
+      </c>
+      <c r="B55" t="s" s="9">
         <v>141</v>
       </c>
-      <c r="B55" t="s" s="9">
+      <c r="C55" t="s" s="9">
         <v>142</v>
-      </c>
-      <c r="C55" t="s" s="9">
-        <v>143</v>
       </c>
       <c r="D55" s="6"/>
       <c r="E55" s="7"/>
     </row>
     <row r="56" ht="20.05" customHeight="1">
       <c r="A56" t="s" s="9">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B56" t="s" s="9">
+        <v>143</v>
+      </c>
+      <c r="C56" t="s" s="9">
         <v>144</v>
-      </c>
-      <c r="C56" t="s" s="9">
-        <v>145</v>
       </c>
       <c r="D56" s="6"/>
       <c r="E56" s="7"/>
     </row>
     <row r="57" ht="20.05" customHeight="1">
       <c r="A57" t="s" s="9">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B57" t="s" s="9">
+        <v>145</v>
+      </c>
+      <c r="C57" t="s" s="9">
         <v>146</v>
-      </c>
-      <c r="C57" t="s" s="9">
-        <v>147</v>
       </c>
       <c r="D57" s="6"/>
       <c r="E57" s="7"/>
     </row>
     <row r="58" ht="20.05" customHeight="1">
       <c r="A58" t="s" s="9">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B58" t="s" s="9">
+        <v>147</v>
+      </c>
+      <c r="C58" t="s" s="9">
         <v>148</v>
-      </c>
-      <c r="C58" t="s" s="9">
-        <v>149</v>
       </c>
       <c r="D58" s="6"/>
       <c r="E58" s="7"/>
     </row>
     <row r="59" ht="32.05" customHeight="1">
       <c r="A59" t="s" s="9">
+        <v>149</v>
+      </c>
+      <c r="B59" t="s" s="9">
         <v>150</v>
       </c>
-      <c r="B59" t="s" s="9">
+      <c r="C59" t="s" s="9">
         <v>151</v>
-      </c>
-      <c r="C59" t="s" s="9">
-        <v>152</v>
       </c>
       <c r="D59" s="6"/>
       <c r="E59" s="7"/>
     </row>
     <row r="60" ht="32.05" customHeight="1">
       <c r="A60" t="s" s="9">
+        <v>152</v>
+      </c>
+      <c r="B60" t="s" s="9">
         <v>153</v>
       </c>
-      <c r="B60" t="s" s="9">
+      <c r="C60" t="s" s="9">
         <v>154</v>
-      </c>
-      <c r="C60" t="s" s="9">
-        <v>155</v>
       </c>
       <c r="D60" s="6"/>
       <c r="E60" s="7"/>
     </row>
     <row r="61" ht="20.05" customHeight="1">
       <c r="A61" t="s" s="9">
+        <v>155</v>
+      </c>
+      <c r="B61" t="s" s="9">
         <v>156</v>
       </c>
-      <c r="B61" t="s" s="9">
+      <c r="C61" t="s" s="9">
         <v>157</v>
-      </c>
-      <c r="C61" t="s" s="9">
-        <v>158</v>
       </c>
       <c r="D61" s="6"/>
       <c r="E61" s="7"/>
     </row>
     <row r="62" ht="20.05" customHeight="1">
       <c r="A62" t="s" s="9">
+        <v>158</v>
+      </c>
+      <c r="B62" t="s" s="9">
         <v>159</v>
       </c>
-      <c r="B62" t="s" s="9">
+      <c r="C62" t="s" s="9">
         <v>160</v>
-      </c>
-      <c r="C62" t="s" s="9">
-        <v>161</v>
       </c>
       <c r="D62" s="10"/>
       <c r="E62" s="11"/>
@@ -3087,10 +3084,10 @@
     <hyperlink ref="C7" r:id="rId6" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dbeec63ad914c973e75c24df"/>
     <hyperlink ref="C8" r:id="rId7" location="" tooltip="" display="https://vinilosargentinos.com/wp-content/uploads/2025/01/y-1.jpg"/>
     <hyperlink ref="C9" r:id="rId8" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273557e06d39588819e7a322817"/>
-    <hyperlink ref="C10" r:id="rId9" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273eb7f16ce83db71362ecb0cb5"/>
-    <hyperlink ref="C11" r:id="rId10" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27314653b83cd7d851accdb5142"/>
-    <hyperlink ref="C12" r:id="rId11" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885"/>
-    <hyperlink ref="C13" r:id="rId12" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab"/>
+    <hyperlink ref="C10" r:id="rId9" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273a2ec3791d9fd51ad343cc885"/>
+    <hyperlink ref="C11" r:id="rId10" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731152471596980e1bba03b6ab"/>
+    <hyperlink ref="C12" r:id="rId11" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273eb7f16ce83db71362ecb0cb5"/>
+    <hyperlink ref="C13" r:id="rId12" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27314653b83cd7d851accdb5142"/>
     <hyperlink ref="C14" r:id="rId13" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27392441ecd34874c2bc4f19144"/>
     <hyperlink ref="C15" r:id="rId14" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2739164bafe9aaa168d93f4816a"/>
     <hyperlink ref="C16" r:id="rId15" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273e21cc1db05580b6f2d2a3b6e"/>
@@ -3119,11 +3116,11 @@
     <hyperlink ref="C39" r:id="rId38" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273bb30191ed1c8b7b14de28135"/>
     <hyperlink ref="C40" r:id="rId39" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b27350db5a166ea23d5d6c4cd387"/>
     <hyperlink ref="C41" r:id="rId40" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273ef221258ca5f3e223937d408"/>
-    <hyperlink ref="C42" r:id="rId41" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87"/>
+    <hyperlink ref="C42" r:id="rId41" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492"/>
     <hyperlink ref="C43" r:id="rId42" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2731351b9b5479c81f76ce7d419"/>
     <hyperlink ref="C44" r:id="rId43" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733025a441495664948b809537"/>
     <hyperlink ref="C45" r:id="rId44" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2737008b56448812cd5b066fe02"/>
-    <hyperlink ref="C46" r:id="rId45" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273986989341960148dac683492"/>
+    <hyperlink ref="C46" r:id="rId45" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273dada67d578bea0b446036e87"/>
     <hyperlink ref="C47" r:id="rId46" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273b57713d0fe3553a087419f8f"/>
     <hyperlink ref="C48" r:id="rId47" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b273056e90910cbaf5c5b892aeba"/>
     <hyperlink ref="C49" r:id="rId48" location="" tooltip="" display="https://i.scdn.co/image/ab67616d0000b2733935c39bea149ac15c83c41a"/>

</xml_diff>